<commit_message>
Monthly event refresh 2026-10
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Events" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Events'!$A$1:$P$161</definedName>
@@ -5188,8 +5188,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr"/>
       <c r="L91" s="3" t="inlineStr">
         <is>
           <t>https://luma.com/34kb3orv</t>
@@ -5208,7 +5206,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -5247,9 +5244,6 @@
           <t>NVIDIA</t>
         </is>
       </c>
-      <c r="I92" t="inlineStr"/>
-      <c r="J92" t="inlineStr"/>
-      <c r="K92" t="inlineStr"/>
       <c r="L92" s="3" t="inlineStr">
         <is>
           <t>https://luma.com/r8sy88tq</t>
@@ -5268,7 +5262,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -5307,9 +5300,6 @@
           <t>Salesforce</t>
         </is>
       </c>
-      <c r="I93" t="inlineStr"/>
-      <c r="J93" t="inlineStr"/>
-      <c r="K93" t="inlineStr"/>
       <c r="L93" s="3" t="inlineStr">
         <is>
           <t>https://luma.com/5ng6bniy</t>
@@ -5328,7 +5318,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -5350,7 +5339,6 @@
           <t>Seattle</t>
         </is>
       </c>
-      <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
           <t>Virtual</t>
@@ -5361,13 +5349,11 @@
           <t>AWS</t>
         </is>
       </c>
-      <c r="I94" t="inlineStr"/>
       <c r="J94" t="inlineStr">
         <is>
           <t>Seattle Business and Technology Meetup Group</t>
         </is>
       </c>
-      <c r="K94" t="inlineStr"/>
       <c r="L94" s="3" t="inlineStr">
         <is>
           <t>https://www.meetup.com/seattle-business-and-technology-meetup-group/events/316816197/</t>
@@ -5386,7 +5372,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5430,8 +5415,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="inlineStr"/>
       <c r="L95" s="3" t="inlineStr">
         <is>
           <t>https://luma.com/agentsinnyc</t>
@@ -5450,7 +5433,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -5472,7 +5454,6 @@
           <t>Seattle</t>
         </is>
       </c>
-      <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
           <t>Virtual</t>
@@ -5493,7 +5474,6 @@
           <t>Microsoft Reactor Redmond</t>
         </is>
       </c>
-      <c r="K96" t="inlineStr"/>
       <c r="L96" s="3" t="inlineStr">
         <is>
           <t>https://www.meetup.com/microsoft-reactor-redmond/events/316854153/</t>
@@ -5512,7 +5492,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -5556,8 +5535,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
       <c r="L97" s="3" t="inlineStr">
         <is>
           <t>https://luma.com/git-sum</t>
@@ -5576,7 +5553,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5613,13 +5589,11 @@
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="I98" t="inlineStr"/>
       <c r="J98" t="inlineStr">
         <is>
           <t>Quadrant Technologies</t>
         </is>
       </c>
-      <c r="K98" t="inlineStr"/>
       <c r="L98" s="3" t="inlineStr">
         <is>
           <t>https://www.meetup.com/real-time-intelligence-using-microsoft-fabric/events/317075539/</t>
@@ -5638,7 +5612,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5682,8 +5655,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J99" t="inlineStr"/>
-      <c r="K99" t="inlineStr"/>
       <c r="L99" s="3" t="inlineStr">
         <is>
           <t>https://luma.com/claude-448g</t>
@@ -5702,7 +5673,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -5749,7 +5719,6 @@
           <t>AWS SBG at University of Washington</t>
         </is>
       </c>
-      <c r="K100" t="inlineStr"/>
       <c r="L100" s="3" t="inlineStr">
         <is>
           <t>https://www.meetup.com/aws-sbg-at-university-of-washington/events/316964535/</t>
@@ -5768,7 +5737,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -5795,7 +5763,6 @@
           <t>Mexico City</t>
         </is>
       </c>
-      <c r="G101" t="inlineStr"/>
       <c r="H101" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -5806,8 +5773,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J101" t="inlineStr"/>
-      <c r="K101" t="inlineStr"/>
       <c r="L101" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/mexicocity27/citylanding/page/cityhome</t>
@@ -5826,7 +5791,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -5848,7 +5812,6 @@
           <t>Seattle</t>
         </is>
       </c>
-      <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
           <t>Virtual</t>
@@ -5859,13 +5822,11 @@
           <t>IBM</t>
         </is>
       </c>
-      <c r="I102" t="inlineStr"/>
       <c r="J102" t="inlineStr">
         <is>
           <t>Data, Cloud and AI in Seattle</t>
         </is>
       </c>
-      <c r="K102" t="inlineStr"/>
       <c r="L102" s="3" t="inlineStr">
         <is>
           <t>https://www.meetup.com/big-data-developers-in-seattle/events/317075384/</t>
@@ -5884,7 +5845,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -5949,7 +5909,6 @@
       <c r="C104" s="2" t="n">
         <v>46331</v>
       </c>
-      <c r="D104" t="inlineStr"/>
       <c r="E104" t="inlineStr">
         <is>
           <t>Bay Area</t>
@@ -5970,9 +5929,6 @@
           <t>SAP</t>
         </is>
       </c>
-      <c r="I104" t="inlineStr"/>
-      <c r="J104" t="inlineStr"/>
-      <c r="K104" t="inlineStr"/>
       <c r="L104" s="3" t="inlineStr">
         <is>
           <t>https://www.eventbrite.co.uk/e/harnessing-data-ai-strategic-technologies-to-drive-business-performance-tickets-2000145093818</t>
@@ -5991,7 +5947,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -6038,7 +5993,6 @@
           <t>Google Developer Group (GDG) Seattle</t>
         </is>
       </c>
-      <c r="K105" t="inlineStr"/>
       <c r="L105" s="3" t="inlineStr">
         <is>
           <t>https://www.meetup.com/gdg-seattle/events/316821635/</t>
@@ -6057,7 +6011,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -6117,7 +6070,6 @@
       <c r="C107" s="2" t="n">
         <v>46338</v>
       </c>
-      <c r="D107" t="inlineStr"/>
       <c r="E107" t="inlineStr">
         <is>
           <t>Seattle</t>
@@ -6138,9 +6090,6 @@
           <t>AWS</t>
         </is>
       </c>
-      <c r="I107" t="inlineStr"/>
-      <c r="J107" t="inlineStr"/>
-      <c r="K107" t="inlineStr"/>
       <c r="L107" s="3" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/saasify-partner-central-agentic-workshop-tickets-2003698327636</t>
@@ -6159,7 +6108,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -6196,13 +6144,11 @@
           <t>Microsoft, Google</t>
         </is>
       </c>
-      <c r="I108" t="inlineStr"/>
       <c r="J108" t="inlineStr">
         <is>
           <t>MaptimeSEA</t>
         </is>
       </c>
-      <c r="K108" t="inlineStr"/>
       <c r="L108" s="3" t="inlineStr">
         <is>
           <t>https://www.meetup.com/maptimesea/events/317097991/</t>
@@ -6221,7 +6167,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -6286,7 +6231,6 @@
       <c r="C110" s="2" t="n">
         <v>46343</v>
       </c>
-      <c r="D110" t="inlineStr"/>
       <c r="E110" t="inlineStr">
         <is>
           <t>Bay Area</t>
@@ -6307,9 +6251,6 @@
           <t>AWS</t>
         </is>
       </c>
-      <c r="I110" t="inlineStr"/>
-      <c r="J110" t="inlineStr"/>
-      <c r="K110" t="inlineStr"/>
       <c r="L110" s="3" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/saasify-partner-central-agentic-workshop-tickets-2003695905391</t>
@@ -6328,7 +6269,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -6406,7 +6346,6 @@
           <t>Washington</t>
         </is>
       </c>
-      <c r="G112" t="inlineStr"/>
       <c r="H112" t="inlineStr">
         <is>
           <t>NVIDIA</t>
@@ -6417,8 +6356,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J112" t="inlineStr"/>
-      <c r="K112" t="inlineStr"/>
       <c r="L112" s="3" t="inlineStr">
         <is>
           <t>https://www.nvidia.com/gtc/events/</t>
@@ -6437,7 +6374,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -6554,22 +6490,16 @@
         <v>46358</v>
       </c>
       <c r="C115" s="2" t="n"/>
-      <c r="D115" t="inlineStr"/>
       <c r="E115" t="inlineStr">
         <is>
           <t>Virtual</t>
         </is>
       </c>
-      <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
         <is>
           <t>Virtual</t>
         </is>
       </c>
-      <c r="H115" t="inlineStr"/>
-      <c r="I115" t="inlineStr"/>
-      <c r="J115" t="inlineStr"/>
-      <c r="K115" t="inlineStr"/>
       <c r="L115" s="3" t="inlineStr">
         <is>
           <t>https://events.channelpronetwork.com/deep-dive-scale-faster-with-zero-trust/</t>
@@ -6588,7 +6518,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -6600,22 +6529,16 @@
         <v>46365</v>
       </c>
       <c r="C116" s="2" t="n"/>
-      <c r="D116" t="inlineStr"/>
       <c r="E116" t="inlineStr">
         <is>
           <t>New York</t>
         </is>
       </c>
-      <c r="F116" t="inlineStr"/>
-      <c r="G116" t="inlineStr"/>
       <c r="H116" t="inlineStr">
         <is>
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="I116" t="inlineStr"/>
-      <c r="J116" t="inlineStr"/>
-      <c r="K116" t="inlineStr"/>
       <c r="L116" s="3" t="inlineStr">
         <is>
           <t>https://themspsummit.com/msp-summit-ai-symposium/</t>
@@ -6634,7 +6557,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -6661,7 +6583,6 @@
           <t>Seattle</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -6672,8 +6593,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J117" t="inlineStr"/>
-      <c r="K117" t="inlineStr"/>
       <c r="L117" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/seattle27/citylanding/page/cityhome</t>
@@ -6692,7 +6611,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -6719,7 +6637,6 @@
           <t>Utrecht</t>
         </is>
       </c>
-      <c r="G118" t="inlineStr"/>
       <c r="H118" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -6730,8 +6647,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J118" t="inlineStr"/>
-      <c r="K118" t="inlineStr"/>
       <c r="L118" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/utrecht27/citylanding/page/cityhome</t>
@@ -6750,7 +6665,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -6777,7 +6691,6 @@
           <t>Toronto</t>
         </is>
       </c>
-      <c r="G119" t="inlineStr"/>
       <c r="H119" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -6788,8 +6701,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J119" t="inlineStr"/>
-      <c r="K119" t="inlineStr"/>
       <c r="L119" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/toronto27/citylanding/page/cityhome</t>
@@ -6808,7 +6719,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -6835,7 +6745,6 @@
           <t>Madrid</t>
         </is>
       </c>
-      <c r="G120" t="inlineStr"/>
       <c r="H120" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -6846,8 +6755,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J120" t="inlineStr"/>
-      <c r="K120" t="inlineStr"/>
       <c r="L120" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/madrid27/citylanding/page/cityhome</t>
@@ -6866,7 +6773,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -6893,7 +6799,6 @@
           <t>Taipei</t>
         </is>
       </c>
-      <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -6904,8 +6809,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J121" t="inlineStr"/>
-      <c r="K121" t="inlineStr"/>
       <c r="L121" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymetaipei/page/notifyme</t>
@@ -6924,7 +6827,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -6951,7 +6853,6 @@
           <t>Chicago</t>
         </is>
       </c>
-      <c r="G122" t="inlineStr"/>
       <c r="H122" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -6962,8 +6863,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J122" t="inlineStr"/>
-      <c r="K122" t="inlineStr"/>
       <c r="L122" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymechicago/page/notifyme</t>
@@ -6982,7 +6881,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -7009,7 +6907,6 @@
           <t>Sydney</t>
         </is>
       </c>
-      <c r="G123" t="inlineStr"/>
       <c r="H123" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -7020,8 +6917,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J123" t="inlineStr"/>
-      <c r="K123" t="inlineStr"/>
       <c r="L123" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymesydney/page/notifyme</t>
@@ -7040,7 +6935,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -7067,7 +6961,6 @@
           <t>Johannesburg</t>
         </is>
       </c>
-      <c r="G124" t="inlineStr"/>
       <c r="H124" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -7078,8 +6971,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J124" t="inlineStr"/>
-      <c r="K124" t="inlineStr"/>
       <c r="L124" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymejoburg/page/notifyme</t>
@@ -7098,7 +6989,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -7125,7 +7015,6 @@
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="G125" t="inlineStr"/>
       <c r="H125" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -7136,8 +7025,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J125" t="inlineStr"/>
-      <c r="K125" t="inlineStr"/>
       <c r="L125" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymemumbai/page/notifyme</t>
@@ -7156,7 +7043,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -7183,7 +7069,6 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G126" t="inlineStr"/>
       <c r="H126" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -7194,8 +7079,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J126" t="inlineStr"/>
-      <c r="K126" t="inlineStr"/>
       <c r="L126" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymebengaluru/page/notifyme</t>
@@ -7214,7 +7097,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -7226,22 +7108,16 @@
         <v>46434</v>
       </c>
       <c r="C127" s="2" t="n"/>
-      <c r="D127" t="inlineStr"/>
       <c r="E127" t="inlineStr">
         <is>
           <t>Virtual</t>
         </is>
       </c>
-      <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
         <is>
           <t>Virtual</t>
         </is>
       </c>
-      <c r="H127" t="inlineStr"/>
-      <c r="I127" t="inlineStr"/>
-      <c r="J127" t="inlineStr"/>
-      <c r="K127" t="inlineStr"/>
       <c r="L127" s="3" t="inlineStr">
         <is>
           <t>https://events.channelpronetwork.com/channelpro-deep-dive-cybersecurity-in-the-age-of-ai/</t>
@@ -7260,7 +7136,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -7287,7 +7162,6 @@
           <t>Milan</t>
         </is>
       </c>
-      <c r="G128" t="inlineStr"/>
       <c r="H128" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -7298,8 +7172,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J128" t="inlineStr"/>
-      <c r="K128" t="inlineStr"/>
       <c r="L128" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymemilan/page/notifyme</t>
@@ -7318,7 +7190,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -7332,18 +7203,11 @@
       <c r="C129" s="2" t="n">
         <v>46455</v>
       </c>
-      <c r="D129" t="inlineStr"/>
       <c r="E129" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="F129" t="inlineStr"/>
-      <c r="G129" t="inlineStr"/>
-      <c r="H129" t="inlineStr"/>
-      <c r="I129" t="inlineStr"/>
-      <c r="J129" t="inlineStr"/>
-      <c r="K129" t="inlineStr"/>
       <c r="L129" s="3" t="inlineStr">
         <is>
           <t>https://event.thechannelco.com/xchange-march/</t>
@@ -7362,7 +7226,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -7396,10 +7259,6 @@
           <t>Virtual</t>
         </is>
       </c>
-      <c r="H130" t="inlineStr"/>
-      <c r="I130" t="inlineStr"/>
-      <c r="J130" t="inlineStr"/>
-      <c r="K130" t="inlineStr"/>
       <c r="L130" s="3" t="inlineStr">
         <is>
           <t>https://channelpartnersconference.com/</t>
@@ -7418,7 +7277,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -7442,8 +7300,6 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="F131" t="inlineStr"/>
-      <c r="G131" t="inlineStr"/>
       <c r="H131" t="inlineStr">
         <is>
           <t>NVIDIA</t>
@@ -7454,8 +7310,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J131" t="inlineStr"/>
-      <c r="K131" t="inlineStr"/>
       <c r="L131" s="3" t="inlineStr">
         <is>
           <t>https://www.nvidia.com/gtc/events/</t>
@@ -7474,7 +7328,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -7501,7 +7354,6 @@
           <t>Stockholm</t>
         </is>
       </c>
-      <c r="G132" t="inlineStr"/>
       <c r="H132" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -7512,8 +7364,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J132" t="inlineStr"/>
-      <c r="K132" t="inlineStr"/>
       <c r="L132" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymestockholm/page/notifyme</t>
@@ -7532,7 +7382,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -7559,7 +7408,6 @@
           <t>New York City</t>
         </is>
       </c>
-      <c r="G133" t="inlineStr"/>
       <c r="H133" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -7570,8 +7418,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J133" t="inlineStr"/>
-      <c r="K133" t="inlineStr"/>
       <c r="L133" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymenyc/page/notifyme</t>
@@ -7590,7 +7436,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -7617,7 +7462,6 @@
           <t>São Paulo</t>
         </is>
       </c>
-      <c r="G134" t="inlineStr"/>
       <c r="H134" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -7628,8 +7472,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J134" t="inlineStr"/>
-      <c r="K134" t="inlineStr"/>
       <c r="L134" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymesaopaulo/page/notifyme</t>
@@ -7648,7 +7490,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -7677,7 +7518,6 @@
           <t>Orlando</t>
         </is>
       </c>
-      <c r="G135" t="inlineStr"/>
       <c r="H135" t="inlineStr">
         <is>
           <t>Oracle</t>
@@ -7688,8 +7528,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J135" t="inlineStr"/>
-      <c r="K135" t="inlineStr"/>
       <c r="L135" s="3" t="inlineStr">
         <is>
           <t>https://www.oracle.com/customer-edge-summit/</t>
@@ -7708,7 +7546,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -7735,7 +7572,6 @@
           <t>Riyadh</t>
         </is>
       </c>
-      <c r="G136" t="inlineStr"/>
       <c r="H136" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -7746,8 +7582,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J136" t="inlineStr"/>
-      <c r="K136" t="inlineStr"/>
       <c r="L136" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymeriyadh/page/notifyme</t>
@@ -7766,7 +7600,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -7788,8 +7621,6 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="F137" t="inlineStr"/>
-      <c r="G137" t="inlineStr"/>
       <c r="H137" t="inlineStr">
         <is>
           <t>Google</t>
@@ -7800,8 +7631,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J137" t="inlineStr"/>
-      <c r="K137" t="inlineStr"/>
       <c r="L137" s="3" t="inlineStr">
         <is>
           <t>https://cloud.google.com/next</t>
@@ -7820,7 +7649,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -7847,7 +7675,6 @@
           <t>Seoul</t>
         </is>
       </c>
-      <c r="G138" t="inlineStr"/>
       <c r="H138" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -7858,8 +7685,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J138" t="inlineStr"/>
-      <c r="K138" t="inlineStr"/>
       <c r="L138" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymeseoul/page/notifyme</t>
@@ -7878,7 +7703,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -7905,7 +7729,6 @@
           <t>Tokyo</t>
         </is>
       </c>
-      <c r="G139" t="inlineStr"/>
       <c r="H139" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -7916,8 +7739,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J139" t="inlineStr"/>
-      <c r="K139" t="inlineStr"/>
       <c r="L139" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymetokyo/page/notifyme</t>
@@ -7936,7 +7757,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -7963,7 +7783,6 @@
           <t>Zurich</t>
         </is>
       </c>
-      <c r="G140" t="inlineStr"/>
       <c r="H140" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -7974,8 +7793,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J140" t="inlineStr"/>
-      <c r="K140" t="inlineStr"/>
       <c r="L140" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymezurich/page/notifyme</t>
@@ -7994,7 +7811,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -8021,7 +7837,6 @@
           <t>Jakarta</t>
         </is>
       </c>
-      <c r="G141" t="inlineStr"/>
       <c r="H141" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -8032,8 +7847,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J141" t="inlineStr"/>
-      <c r="K141" t="inlineStr"/>
       <c r="L141" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymejakarta/page/notifyme</t>
@@ -8052,7 +7865,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -8079,7 +7891,6 @@
           <t>Miami</t>
         </is>
       </c>
-      <c r="G142" t="inlineStr"/>
       <c r="H142" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -8090,8 +7901,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J142" t="inlineStr"/>
-      <c r="K142" t="inlineStr"/>
       <c r="L142" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymemiami/page/notifyme</t>
@@ -8110,7 +7919,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -8137,7 +7945,6 @@
           <t>Copenhagen</t>
         </is>
       </c>
-      <c r="G143" t="inlineStr"/>
       <c r="H143" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -8148,8 +7955,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J143" t="inlineStr"/>
-      <c r="K143" t="inlineStr"/>
       <c r="L143" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymecopenhagen/page/notifyme</t>
@@ -8168,7 +7973,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -8195,7 +7999,6 @@
           <t>Montreal</t>
         </is>
       </c>
-      <c r="G144" t="inlineStr"/>
       <c r="H144" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -8206,8 +8009,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J144" t="inlineStr"/>
-      <c r="K144" t="inlineStr"/>
       <c r="L144" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymemontreal/page/notifyme</t>
@@ -8226,7 +8027,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -8253,7 +8053,6 @@
           <t>Brussels</t>
         </is>
       </c>
-      <c r="G145" t="inlineStr"/>
       <c r="H145" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -8264,8 +8063,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J145" t="inlineStr"/>
-      <c r="K145" t="inlineStr"/>
       <c r="L145" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymebrussels/page/notifyme</t>
@@ -8284,7 +8081,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -8296,22 +8092,16 @@
         <v>46539</v>
       </c>
       <c r="C146" s="2" t="n"/>
-      <c r="D146" t="inlineStr"/>
       <c r="E146" t="inlineStr">
         <is>
           <t>Virtual</t>
         </is>
       </c>
-      <c r="F146" t="inlineStr"/>
       <c r="G146" t="inlineStr">
         <is>
           <t>Virtual</t>
         </is>
       </c>
-      <c r="H146" t="inlineStr"/>
-      <c r="I146" t="inlineStr"/>
-      <c r="J146" t="inlineStr"/>
-      <c r="K146" t="inlineStr"/>
       <c r="L146" s="3" t="inlineStr">
         <is>
           <t>https://events.channelpronetwork.com/channelpro-deep-dive-the-most-profitable-cybersecurity-services-in-2027/</t>
@@ -8330,7 +8120,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -8357,7 +8146,6 @@
           <t>Houston</t>
         </is>
       </c>
-      <c r="G147" t="inlineStr"/>
       <c r="H147" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -8368,8 +8156,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J147" t="inlineStr"/>
-      <c r="K147" t="inlineStr"/>
       <c r="L147" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymehouston/page/notifyme</t>
@@ -8388,7 +8174,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -8415,7 +8200,6 @@
           <t>Tel Aviv</t>
         </is>
       </c>
-      <c r="G148" t="inlineStr"/>
       <c r="H148" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -8426,8 +8210,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J148" t="inlineStr"/>
-      <c r="K148" t="inlineStr"/>
       <c r="L148" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymetelaviv/page/notifyme</t>
@@ -8446,7 +8228,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -8470,7 +8251,6 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr">
         <is>
           <t>Hybrid</t>
@@ -8514,7 +8294,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -8538,8 +8317,6 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="F150" t="inlineStr"/>
-      <c r="G150" t="inlineStr"/>
       <c r="H150" t="inlineStr">
         <is>
           <t>Snowflake, Anthropic</t>
@@ -8550,8 +8327,6 @@
           <t>Host, Speaker</t>
         </is>
       </c>
-      <c r="J150" t="inlineStr"/>
-      <c r="K150" t="inlineStr"/>
       <c r="L150" s="3" t="inlineStr">
         <is>
           <t>https://www.snowflake.com/en/summit/</t>
@@ -8570,7 +8345,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -8597,7 +8371,6 @@
           <t>Atlanta</t>
         </is>
       </c>
-      <c r="G151" t="inlineStr"/>
       <c r="H151" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -8608,8 +8381,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J151" t="inlineStr"/>
-      <c r="K151" t="inlineStr"/>
       <c r="L151" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymeatlanta/page/notifyme</t>
@@ -8628,7 +8399,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -8652,8 +8422,6 @@
           <t>Bay Area</t>
         </is>
       </c>
-      <c r="F152" t="inlineStr"/>
-      <c r="G152" t="inlineStr"/>
       <c r="H152" t="inlineStr">
         <is>
           <t>Databricks</t>
@@ -8664,8 +8432,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J152" t="inlineStr"/>
-      <c r="K152" t="inlineStr"/>
       <c r="L152" s="3" t="inlineStr">
         <is>
           <t>https://www.databricks.com/dataaisummit/agenda</t>
@@ -8684,7 +8450,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -8711,7 +8476,6 @@
           <t>Osaka</t>
         </is>
       </c>
-      <c r="G153" t="inlineStr"/>
       <c r="H153" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -8722,8 +8486,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J153" t="inlineStr"/>
-      <c r="K153" t="inlineStr"/>
       <c r="L153" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymeosaka/page/notifyme</t>
@@ -8742,7 +8504,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -8754,22 +8515,16 @@
         <v>46623</v>
       </c>
       <c r="C154" s="2" t="n"/>
-      <c r="D154" t="inlineStr"/>
       <c r="E154" t="inlineStr">
         <is>
           <t>Virtual</t>
         </is>
       </c>
-      <c r="F154" t="inlineStr"/>
       <c r="G154" t="inlineStr">
         <is>
           <t>Virtual</t>
         </is>
       </c>
-      <c r="H154" t="inlineStr"/>
-      <c r="I154" t="inlineStr"/>
-      <c r="J154" t="inlineStr"/>
-      <c r="K154" t="inlineStr"/>
       <c r="L154" s="3" t="inlineStr">
         <is>
           <t>https://events.channelpronetwork.com/channelpro-deep-dive-where-the-next-wave-of-msp-revenue-is-coming-from/</t>
@@ -8788,7 +8543,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -8810,8 +8564,6 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="F155" t="inlineStr"/>
-      <c r="G155" t="inlineStr"/>
       <c r="H155" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -8822,8 +8574,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J155" t="inlineStr"/>
-      <c r="K155" t="inlineStr"/>
       <c r="L155" s="3" t="inlineStr">
         <is>
           <t>https://www.techcon365.com/Seattle/</t>
@@ -8842,7 +8592,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -8866,8 +8615,6 @@
           <t>Bay Area</t>
         </is>
       </c>
-      <c r="F156" t="inlineStr"/>
-      <c r="G156" t="inlineStr"/>
       <c r="H156" t="inlineStr">
         <is>
           <t>Salesforce</t>
@@ -8878,8 +8625,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J156" t="inlineStr"/>
-      <c r="K156" t="inlineStr"/>
       <c r="L156" s="3" t="inlineStr">
         <is>
           <t>https://www.salesforce.com/dreamforce/</t>
@@ -8898,7 +8643,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -8912,18 +8656,11 @@
       <c r="C157" s="2" t="n">
         <v>46659</v>
       </c>
-      <c r="D157" t="inlineStr"/>
       <c r="E157" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="F157" t="inlineStr"/>
-      <c r="G157" t="inlineStr"/>
-      <c r="H157" t="inlineStr"/>
-      <c r="I157" t="inlineStr"/>
-      <c r="J157" t="inlineStr"/>
-      <c r="K157" t="inlineStr"/>
       <c r="L157" s="3" t="inlineStr">
         <is>
           <t>https://technology.informaengage.com/msps27-get-notified</t>
@@ -8942,7 +8679,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -8966,8 +8702,6 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="F158" t="inlineStr"/>
-      <c r="G158" t="inlineStr"/>
       <c r="H158" t="inlineStr">
         <is>
           <t>Workday</t>
@@ -8978,8 +8712,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J158" t="inlineStr"/>
-      <c r="K158" t="inlineStr"/>
       <c r="L158" s="3" t="inlineStr">
         <is>
           <t>https://rising.workday.com/us.html</t>
@@ -8998,7 +8730,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -9022,8 +8753,6 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="F159" t="inlineStr"/>
-      <c r="G159" t="inlineStr"/>
       <c r="H159" t="inlineStr">
         <is>
           <t>Okta</t>
@@ -9034,8 +8763,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J159" t="inlineStr"/>
-      <c r="K159" t="inlineStr"/>
       <c r="L159" s="3" t="inlineStr">
         <is>
           <t>https://www.okta.com/oktane/on-demand/</t>
@@ -9054,7 +8781,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -9066,22 +8792,16 @@
         <v>46679</v>
       </c>
       <c r="C160" s="2" t="n"/>
-      <c r="D160" t="inlineStr"/>
       <c r="E160" t="inlineStr">
         <is>
           <t>Virtual</t>
         </is>
       </c>
-      <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr">
         <is>
           <t>Virtual</t>
         </is>
       </c>
-      <c r="H160" t="inlineStr"/>
-      <c r="I160" t="inlineStr"/>
-      <c r="J160" t="inlineStr"/>
-      <c r="K160" t="inlineStr"/>
       <c r="L160" s="3" t="inlineStr">
         <is>
           <t>https://events.channelpronetwork.com/channelpro-deep-dive-the-ai-powered-msp/</t>
@@ -9100,7 +8820,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -9129,7 +8848,6 @@
           <t>Las Vegas</t>
         </is>
       </c>
-      <c r="G161" t="inlineStr"/>
       <c r="H161" t="inlineStr">
         <is>
           <t>Oracle</t>
@@ -9140,8 +8858,6 @@
           <t>Host, Speaker</t>
         </is>
       </c>
-      <c r="J161" t="inlineStr"/>
-      <c r="K161" t="inlineStr"/>
       <c r="L161" s="3" t="inlineStr">
         <is>
           <t>https://www.oracle.com/ai-world/</t>
@@ -9160,7 +8876,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="P161" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:P161"/>

</xml_diff>

<commit_message>
Make Events a real Excel Table and publish an ISO-dated tracker.csv
Power Query showed the date columns as serial numbers; the CSV gives it unambiguous date text and the Table gives typed columns.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TLMW817qEmLPfhM4KiByCq
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -1,17 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Events" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Events'!$A$1:$P$161</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -145,6 +143,31 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Events" displayName="Events" ref="A1:P161" headerRowCount="1">
+  <autoFilter ref="A1:P161"/>
+  <tableColumns count="16">
+    <tableColumn id="1" name="Name"/>
+    <tableColumn id="2" name="Date"/>
+    <tableColumn id="3" name="End Date"/>
+    <tableColumn id="4" name="Organiser/Host"/>
+    <tableColumn id="5" name="Region"/>
+    <tableColumn id="6" name="City"/>
+    <tableColumn id="7" name="Format"/>
+    <tableColumn id="8" name="Companies Attending"/>
+    <tableColumn id="9" name="Role"/>
+    <tableColumn id="10" name="Named Speakers"/>
+    <tableColumn id="11" name="Cost"/>
+    <tableColumn id="12" name="URL"/>
+    <tableColumn id="13" name="Source"/>
+    <tableColumn id="14" name="Date Added"/>
+    <tableColumn id="15" name="Status"/>
+    <tableColumn id="16" name="Notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8878,7 +8901,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P161"/>
   <dataValidations count="1">
     <dataValidation sqref="O2:O5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"New,Attending,Skip"</formula1>
@@ -9024,5 +9046,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L161" r:id="rId137"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId138"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
A named venue/city overrides a mislabelled virtual attendance mode
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TLMW817qEmLPfhM4KiByCq
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -146,8 +146,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Events" displayName="Events" ref="A1:P68" headerRowCount="1">
-  <autoFilter ref="A1:P68"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Events" displayName="Events" ref="A1:P67" headerRowCount="1">
+  <autoFilter ref="A1:P67"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Name"/>
     <tableColumn id="2" name="Date"/>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P68"/>
+  <dimension ref="A1:P67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -3728,47 +3728,49 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Channel Partners Conference &amp; Expo 2027</t>
+          <t>Microsoft AI Tour - New York City</t>
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>46461</v>
-      </c>
-      <c r="C59" s="2" t="n">
         <v>46464</v>
       </c>
+      <c r="C59" s="2" t="n"/>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Informa Group PLC</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Virtual</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>The Venetian</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
       <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr"/>
       <c r="L59" s="3" t="inlineStr">
         <is>
-          <t>https://channelpartnersconference.com/</t>
+          <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymenyc/page/notifyme</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>Channel Partners Conference</t>
+          <t>Microsoft AI Tour</t>
         </is>
       </c>
       <c r="N59" s="2" t="n">
@@ -3784,49 +3786,41 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Microsoft AI Tour - New York City</t>
+          <t>ChannelPro DEEP DIVE: Perfecting Your Tool Stack</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>46464</v>
+        <v>46483</v>
       </c>
       <c r="C60" s="2" t="n"/>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>ChannelPro Network</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>New York</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>New York City</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>Host</t>
-        </is>
-      </c>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
       <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr"/>
       <c r="L60" s="3" t="inlineStr">
         <is>
-          <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymenyc/page/notifyme</t>
+          <t>https://events.channelpronetwork.com/channelpro-deep-dive-perfecting-your-tool-stack/</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>Microsoft AI Tour</t>
+          <t>Channel Pro Network</t>
         </is>
       </c>
       <c r="N60" s="2" t="n">
@@ -3842,11 +3836,11 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ChannelPro DEEP DIVE: Perfecting Your Tool Stack</t>
+          <t>ChannelPro DEEP DIVE: The Most Profitable Cybersecurity Services in 2027</t>
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>46483</v>
+        <v>46539</v>
       </c>
       <c r="C61" s="2" t="n"/>
       <c r="D61" t="inlineStr">
@@ -3871,7 +3865,7 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" s="3" t="inlineStr">
         <is>
-          <t>https://events.channelpronetwork.com/channelpro-deep-dive-perfecting-your-tool-stack/</t>
+          <t>https://events.channelpronetwork.com/channelpro-deep-dive-the-most-profitable-cybersecurity-services-in-2027/</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
@@ -3892,41 +3886,49 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ChannelPro DEEP DIVE: The Most Profitable Cybersecurity Services in 2027</t>
+          <t>Microsoft AI Tour - Houston</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>46539</v>
+        <v>46540</v>
       </c>
       <c r="C62" s="2" t="n"/>
       <c r="D62" t="inlineStr">
         <is>
-          <t>ChannelPro Network</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
+          <t>Texas</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
       <c r="J62" t="inlineStr"/>
       <c r="K62" t="inlineStr"/>
       <c r="L62" s="3" t="inlineStr">
         <is>
-          <t>https://events.channelpronetwork.com/channelpro-deep-dive-the-most-profitable-cybersecurity-services-in-2027/</t>
+          <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymehouston/page/notifyme</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>Channel Pro Network</t>
+          <t>Microsoft AI Tour</t>
         </is>
       </c>
       <c r="N62" s="2" t="n">
@@ -3942,32 +3944,30 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Microsoft AI Tour - Houston</t>
+          <t>Databricks Data+AI Summit 2027</t>
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>46540</v>
-      </c>
-      <c r="C63" s="2" t="n"/>
+        <v>46559</v>
+      </c>
+      <c r="C63" s="2" t="n">
+        <v>46562</v>
+      </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Texas</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>Houston</t>
-        </is>
-      </c>
+          <t>Bay Area</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3979,12 +3979,12 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" s="3" t="inlineStr">
         <is>
-          <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymehouston/page/notifyme</t>
+          <t>https://www.databricks.com/dataaisummit/agenda</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>Microsoft AI Tour</t>
+          <t>Databricks Data+AI Summit</t>
         </is>
       </c>
       <c r="N63" s="2" t="n">
@@ -4000,47 +4000,41 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Databricks Data+AI Summit 2027</t>
+          <t>ChannelPro DEEP DIVE: Where the Next Wave of MSP Revenue Is Coming From</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>46559</v>
-      </c>
-      <c r="C64" s="2" t="n">
-        <v>46562</v>
-      </c>
+        <v>46623</v>
+      </c>
+      <c r="C64" s="2" t="n"/>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>ChannelPro Network</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Bay Area</t>
+          <t>Virtual</t>
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>Databricks</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>Host</t>
-        </is>
-      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
       <c r="J64" t="inlineStr"/>
       <c r="K64" t="inlineStr"/>
       <c r="L64" s="3" t="inlineStr">
         <is>
-          <t>https://www.databricks.com/dataaisummit/agenda</t>
+          <t>https://events.channelpronetwork.com/channelpro-deep-dive-where-the-next-wave-of-msp-revenue-is-coming-from/</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>Databricks Data+AI Summit</t>
+          <t>Channel Pro Network</t>
         </is>
       </c>
       <c r="N64" s="2" t="n">
@@ -4056,13 +4050,15 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ChannelPro DEEP DIVE: Where the Next Wave of MSP Revenue Is Coming From</t>
+          <t>2027 ChannelPro DEFEND: Dallas</t>
         </is>
       </c>
       <c r="B65" s="2" t="n">
-        <v>46623</v>
-      </c>
-      <c r="C65" s="2" t="n"/>
+        <v>46644</v>
+      </c>
+      <c r="C65" s="2" t="n">
+        <v>46645</v>
+      </c>
       <c r="D65" t="inlineStr">
         <is>
           <t>ChannelPro Network</t>
@@ -4070,22 +4066,18 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Virtual</t>
+          <t>Texas</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
+      <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr"/>
       <c r="J65" t="inlineStr"/>
       <c r="K65" t="inlineStr"/>
       <c r="L65" s="3" t="inlineStr">
         <is>
-          <t>https://events.channelpronetwork.com/channelpro-deep-dive-where-the-next-wave-of-msp-revenue-is-coming-from/</t>
+          <t>https://events.channelpronetwork.com/2027-channelpro-defend-dallas/</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
@@ -4106,39 +4098,47 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2027 ChannelPro DEFEND: Dallas</t>
+          <t>Dreamforce 2027</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>46644</v>
+        <v>46651</v>
       </c>
       <c r="C66" s="2" t="n">
-        <v>46645</v>
+        <v>46653</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>ChannelPro Network</t>
+          <t>Salesforce</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Texas</t>
+          <t>Bay Area</t>
         </is>
       </c>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Salesforce</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
       <c r="J66" t="inlineStr"/>
       <c r="K66" t="inlineStr"/>
       <c r="L66" s="3" t="inlineStr">
         <is>
-          <t>https://events.channelpronetwork.com/2027-channelpro-defend-dallas/</t>
+          <t>https://www.salesforce.com/dreamforce/</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>Channel Pro Network</t>
+          <t>Dreamforce</t>
         </is>
       </c>
       <c r="N66" s="2" t="n">
@@ -4154,47 +4154,41 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Dreamforce 2027</t>
+          <t>ChannelPro DEEP DIVE: The AI-Powered MSP</t>
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>46651</v>
-      </c>
-      <c r="C67" s="2" t="n">
-        <v>46653</v>
-      </c>
+        <v>46679</v>
+      </c>
+      <c r="C67" s="2" t="n"/>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Salesforce</t>
+          <t>ChannelPro Network</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Bay Area</t>
+          <t>Virtual</t>
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>Salesforce</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>Host</t>
-        </is>
-      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
       <c r="J67" t="inlineStr"/>
       <c r="K67" t="inlineStr"/>
       <c r="L67" s="3" t="inlineStr">
         <is>
-          <t>https://www.salesforce.com/dreamforce/</t>
+          <t>https://events.channelpronetwork.com/channelpro-deep-dive-the-ai-powered-msp/</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>Dreamforce</t>
+          <t>Channel Pro Network</t>
         </is>
       </c>
       <c r="N67" s="2" t="n">
@@ -4206,56 +4200,6 @@
         </is>
       </c>
       <c r="P67" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>ChannelPro DEEP DIVE: The AI-Powered MSP</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="n">
-        <v>46679</v>
-      </c>
-      <c r="C68" s="2" t="n"/>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>ChannelPro Network</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr"/>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" s="3" t="inlineStr">
-        <is>
-          <t>https://events.channelpronetwork.com/channelpro-deep-dive-the-ai-powered-msp/</t>
-        </is>
-      </c>
-      <c r="M68" t="inlineStr">
-        <is>
-          <t>Channel Pro Network</t>
-        </is>
-      </c>
-      <c r="N68" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O68" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="P68" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -4313,11 +4257,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L65" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L66" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L67" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L68" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId51"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId50"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Remove Date Added, Status and Notes columns
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TLMW817qEmLPfhM4KiByCq
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -146,9 +146,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Events" displayName="Events" ref="A1:P67" headerRowCount="1">
-  <autoFilter ref="A1:P67"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Events" displayName="Events" ref="A1:M68" headerRowCount="1">
+  <autoFilter ref="A1:M68"/>
+  <tableColumns count="13">
     <tableColumn id="1" name="Name"/>
     <tableColumn id="2" name="Date"/>
     <tableColumn id="3" name="End Date"/>
@@ -162,9 +162,6 @@
     <tableColumn id="11" name="Cost"/>
     <tableColumn id="12" name="URL"/>
     <tableColumn id="13" name="Source"/>
-    <tableColumn id="14" name="Date Added"/>
-    <tableColumn id="15" name="Status"/>
-    <tableColumn id="16" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -459,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P67"/>
+  <dimension ref="A1:M68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -475,9 +472,6 @@
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="45" customWidth="1" min="12" max="12"/>
     <col width="26" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="30" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -546,21 +540,6 @@
           <t>Source</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Date Added</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -612,14 +591,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N2" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -658,14 +629,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N3" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -717,14 +680,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N4" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -776,14 +731,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N5" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -835,14 +782,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N6" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -896,14 +835,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N7" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -955,14 +886,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N8" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1001,14 +924,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N9" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1060,14 +975,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N10" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1109,14 +1016,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N11" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1168,14 +1067,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N12" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1229,14 +1120,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N13" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1290,14 +1173,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N14" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1341,14 +1216,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N15" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1402,14 +1269,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N16" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1453,14 +1312,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N17" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1512,14 +1363,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N18" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1573,14 +1416,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N19" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1629,14 +1464,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N20" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1690,14 +1517,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N21" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1746,14 +1565,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N22" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1802,14 +1613,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N23" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1856,14 +1659,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N24" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1910,14 +1705,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N25" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1964,14 +1751,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N26" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2018,14 +1797,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N27" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2079,14 +1850,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N28" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2135,14 +1898,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N29" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2196,14 +1951,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N30" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2250,14 +1997,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N31" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2304,14 +2043,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N32" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2358,14 +2089,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N33" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2414,14 +2137,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N34" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2470,14 +2185,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N35" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2526,14 +2233,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N36" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2580,14 +2279,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N37" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2634,14 +2325,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N38" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O38" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2685,14 +2368,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N39" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2739,14 +2414,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N40" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O40" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2790,14 +2457,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N41" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O41" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2844,14 +2503,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N42" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O42" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2900,14 +2551,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N43" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O43" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2949,14 +2592,6 @@
       <c r="M44" t="inlineStr">
         <is>
           <t>Legacy tracker 2026</t>
-        </is>
-      </c>
-      <c r="N44" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O44" t="inlineStr">
-        <is>
-          <t>New</t>
         </is>
       </c>
     </row>
@@ -3014,15 +2649,6 @@
           <t>Luma NYC</t>
         </is>
       </c>
-      <c r="N45" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O45" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="P45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3071,14 +2697,6 @@
           <t>Legacy tracker 2026</t>
         </is>
       </c>
-      <c r="N46" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O46" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3120,14 +2738,6 @@
       <c r="M47" t="inlineStr">
         <is>
           <t>Legacy tracker 2026</t>
-        </is>
-      </c>
-      <c r="N47" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O47" t="inlineStr">
-        <is>
-          <t>New</t>
         </is>
       </c>
     </row>
@@ -3177,85 +2787,77 @@
           <t>Eventbrite Seattle - AWS/Microsoft/Google</t>
         </is>
       </c>
-      <c r="N48" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O48" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="P48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Microsoft Ignite 2026</t>
+          <t>Identity, AI &amp; Cybersecurity: Securing the Enterprise in an Agentic World</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>46343</v>
-      </c>
-      <c r="C49" s="2" t="n">
-        <v>46346</v>
-      </c>
+        <v>46339</v>
+      </c>
+      <c r="C49" s="2" t="n"/>
       <c r="D49" t="inlineStr">
         <is>
+          <t>Seattle Data, AI &amp; Security</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Seattle</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Bellevue</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Bay Area</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>San Francisco</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>In-person</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Seattle Data, AI &amp; Security</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr"/>
       <c r="L49" s="3" t="inlineStr">
         <is>
-          <t>https://ignite.microsoft.com/en-US/home</t>
+          <t>https://www.meetup.com/seattledataaiandsecurity/events/316481475/</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>Legacy tracker 2026</t>
-        </is>
-      </c>
-      <c r="N49" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O49" t="inlineStr">
-        <is>
-          <t>New</t>
+          <t>Meetup Seattle - AWS</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>SaaSify Partner Central Agentic Workshop</t>
+          <t>Microsoft Ignite 2026</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
         <v>46343</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>46343</v>
-      </c>
-      <c r="D50" t="inlineStr"/>
+        <v>46346</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
       <c r="E50" t="inlineStr">
         <is>
           <t>Bay Area</t>
@@ -3273,47 +2875,33 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>AWS</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
+          <t>Microsoft</t>
+        </is>
+      </c>
       <c r="L50" s="3" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/saasify-partner-central-agentic-workshop-tickets-2003695905391</t>
+          <t>https://ignite.microsoft.com/en-US/home</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>Eventbrite SF - cloud partner</t>
-        </is>
-      </c>
-      <c r="N50" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O50" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="P50" t="inlineStr"/>
+          <t>Legacy tracker 2026</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Cloudflare Immerse</t>
+          <t>SaaSify Partner Central Agentic Workshop</t>
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>46346</v>
-      </c>
-      <c r="C51" s="2" t="n"/>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Cloudflare</t>
-        </is>
-      </c>
+        <v>46343</v>
+      </c>
+      <c r="C51" s="2" t="n">
+        <v>46343</v>
+      </c>
+      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
           <t>Bay Area</t>
@@ -3321,7 +2909,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Bay Area</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3331,51 +2919,46 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Cloudflare</t>
-        </is>
-      </c>
+          <t>AWS</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
       <c r="L51" s="3" t="inlineStr">
         <is>
-          <t>https://fieldmarketing.www.cloudflare.com/cloudflareimmersebayarea?_gl=1*1ge1j1x*_gcl_au*MjMxOTM0MjE4LjE3NTkzNjYwMjI.*_ga*ZmI3OTU3NjUtZDkyOC00M2I3LWJiOGYtNzQ5ZjJlZGUxYWFm*_ga_SQCRB0TXZW*czE3NjU0NjEwMDIkbzMkZzEkdDE3NjU0NjEwNTkkajMkbDAkaDAkZHVGb1hkWDJpQmU2OUExYjJSSl92c2xTbkxWQURDZTlUSWc.</t>
+          <t>https://www.eventbrite.com/e/saasify-partner-central-agentic-workshop-tickets-2003695905391</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>Legacy tracker 2026</t>
-        </is>
-      </c>
-      <c r="N51" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O51" t="inlineStr">
-        <is>
-          <t>New</t>
+          <t>Eventbrite SF - cloud partner</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Gartner / Evanta Seattle CIO Community Executive Summit</t>
+          <t>Cloudflare Immerse</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>46357</v>
+        <v>46346</v>
       </c>
       <c r="C52" s="2" t="n"/>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Google Cloud / Cloudflare / Dynatrace</t>
+          <t>Cloudflare</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Bay Area</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Bay Area</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3385,140 +2968,111 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Google, Dynatrace, Cloudflare</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>Invite/application-based; no public attendee fee</t>
+          <t>Cloudflare</t>
+        </is>
+      </c>
+      <c r="L52" s="3" t="inlineStr">
+        <is>
+          <t>https://fieldmarketing.www.cloudflare.com/cloudflareimmersebayarea?_gl=1*1ge1j1x*_gcl_au*MjMxOTM0MjE4LjE3NTkzNjYwMjI.*_ga*ZmI3OTU3NjUtZDkyOC00M2I3LWJiOGYtNzQ5ZjJlZGUxYWFm*_ga_SQCRB0TXZW*czE3NjU0NjEwMDIkbzMkZzEkdDE3NjU0NjEwNTkkajMkbDAkaDAkZHVGb1hkWDJpQmU2OUExYjJSSl92c2xTbkxWQURDZTlUSWc.</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
         <is>
           <t>Legacy tracker 2026</t>
-        </is>
-      </c>
-      <c r="N52" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O52" t="inlineStr">
-        <is>
-          <t>New</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>MSP Summit: AI Symposium</t>
+          <t>Gartner / Evanta Seattle CIO Community Executive Summit</t>
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>46365</v>
+        <v>46357</v>
       </c>
       <c r="C53" s="2" t="n"/>
-      <c r="D53" t="inlineStr"/>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Google Cloud / Cloudflare / Dynatrace</t>
+        </is>
+      </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>New York</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
+          <t>Seattle</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Seattle</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" s="3" t="inlineStr">
-        <is>
-          <t>https://themspsummit.com/msp-summit-ai-symposium/</t>
+          <t>Google, Dynatrace, Cloudflare</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Invite/application-based; no public attendee fee</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>MSP Summit / events calendar</t>
-        </is>
-      </c>
-      <c r="N53" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O53" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="P53" t="inlineStr"/>
+          <t>Legacy tracker 2026</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Microsoft AI Tour - Seattle</t>
+          <t>MSP Summit: AI Symposium</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
         <v>46365</v>
       </c>
       <c r="C54" s="2" t="n"/>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
+      <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Seattle</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>Seattle</t>
-        </is>
-      </c>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>Host</t>
-        </is>
-      </c>
+      <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr"/>
       <c r="K54" t="inlineStr"/>
       <c r="L54" s="3" t="inlineStr">
         <is>
-          <t>https://aitour.microsoft.com/flow/microsoft/seattle27/citylanding/page/cityhome</t>
+          <t>https://themspsummit.com/msp-summit-ai-symposium/</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>Microsoft AI Tour</t>
-        </is>
-      </c>
-      <c r="N54" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O54" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="P54" t="inlineStr"/>
+          <t>MSP Summit / events calendar</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Microsoft AI Tour - Mumbai</t>
+          <t>Microsoft AI Tour - Seattle</t>
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>46428</v>
+        <v>46365</v>
       </c>
       <c r="C55" s="2" t="n"/>
       <c r="D55" t="inlineStr">
@@ -3528,12 +3082,12 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Mumbai</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="G55" t="inlineStr"/>
@@ -3551,7 +3105,7 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" s="3" t="inlineStr">
         <is>
-          <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymemumbai/page/notifyme</t>
+          <t>https://aitour.microsoft.com/flow/microsoft/seattle27/citylanding/page/cityhome</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
@@ -3559,24 +3113,15 @@
           <t>Microsoft AI Tour</t>
         </is>
       </c>
-      <c r="N55" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O55" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="P55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Microsoft AI Tour - Bengaluru</t>
+          <t>Microsoft AI Tour - Mumbai</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>46433</v>
+        <v>46428</v>
       </c>
       <c r="C56" s="2" t="n"/>
       <c r="D56" t="inlineStr">
@@ -3591,7 +3136,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Mumbai</t>
         </is>
       </c>
       <c r="G56" t="inlineStr"/>
@@ -3609,7 +3154,7 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" s="3" t="inlineStr">
         <is>
-          <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymebengaluru/page/notifyme</t>
+          <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymemumbai/page/notifyme</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
@@ -3617,230 +3162,193 @@
           <t>Microsoft AI Tour</t>
         </is>
       </c>
-      <c r="N56" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O56" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="P56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ChannelPro DEEP DIVE: Cybersecurity in the Age of AI</t>
+          <t>Microsoft AI Tour - Bengaluru</t>
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>46434</v>
+        <v>46433</v>
       </c>
       <c r="C57" s="2" t="n"/>
       <c r="D57" t="inlineStr">
         <is>
-          <t>ChannelPro Network</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
       <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr"/>
       <c r="L57" s="3" t="inlineStr">
         <is>
-          <t>https://events.channelpronetwork.com/channelpro-deep-dive-cybersecurity-in-the-age-of-ai/</t>
+          <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymebengaluru/page/notifyme</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>Channel Pro Network</t>
-        </is>
-      </c>
-      <c r="N57" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O57" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="P57" t="inlineStr"/>
+          <t>Microsoft AI Tour</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Xchange 2027</t>
+          <t>ChannelPro DEEP DIVE: Cybersecurity in the Age of AI</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>46453</v>
-      </c>
-      <c r="C58" s="2" t="n">
-        <v>46455</v>
-      </c>
+        <v>46434</v>
+      </c>
+      <c r="C58" s="2" t="n"/>
       <c r="D58" t="inlineStr">
         <is>
-          <t>The Channel Company</t>
+          <t>ChannelPro Network</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Texas</t>
+          <t>Virtual</t>
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
       <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr"/>
       <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr"/>
       <c r="L58" s="3" t="inlineStr">
         <is>
-          <t>https://event.thechannelco.com/xchange-march/</t>
+          <t>https://events.channelpronetwork.com/channelpro-deep-dive-cybersecurity-in-the-age-of-ai/</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>Xchange (The Channel Co)</t>
-        </is>
-      </c>
-      <c r="N58" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O58" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="P58" t="inlineStr"/>
+          <t>Channel Pro Network</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Microsoft AI Tour - New York City</t>
+          <t>Xchange 2027</t>
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>46464</v>
-      </c>
-      <c r="C59" s="2" t="n"/>
+        <v>46453</v>
+      </c>
+      <c r="C59" s="2" t="n">
+        <v>46455</v>
+      </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>The Channel Company</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>New York</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>New York City</t>
-        </is>
-      </c>
+          <t>Texas</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>Host</t>
-        </is>
-      </c>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr"/>
       <c r="L59" s="3" t="inlineStr">
         <is>
-          <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymenyc/page/notifyme</t>
+          <t>https://event.thechannelco.com/xchange-march/</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>Microsoft AI Tour</t>
-        </is>
-      </c>
-      <c r="N59" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O59" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="P59" t="inlineStr"/>
+          <t>Xchange (The Channel Co)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ChannelPro DEEP DIVE: Perfecting Your Tool Stack</t>
+          <t>Microsoft AI Tour - New York City</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>46483</v>
+        <v>46464</v>
       </c>
       <c r="C60" s="2" t="n"/>
       <c r="D60" t="inlineStr">
         <is>
-          <t>ChannelPro Network</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
       <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr"/>
       <c r="L60" s="3" t="inlineStr">
         <is>
-          <t>https://events.channelpronetwork.com/channelpro-deep-dive-perfecting-your-tool-stack/</t>
+          <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymenyc/page/notifyme</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>Channel Pro Network</t>
-        </is>
-      </c>
-      <c r="N60" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O60" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="P60" t="inlineStr"/>
+          <t>Microsoft AI Tour</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ChannelPro DEEP DIVE: The Most Profitable Cybersecurity Services in 2027</t>
+          <t>ChannelPro DEEP DIVE: Perfecting Your Tool Stack</t>
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>46539</v>
+        <v>46483</v>
       </c>
       <c r="C61" s="2" t="n"/>
       <c r="D61" t="inlineStr">
@@ -3865,7 +3373,7 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" s="3" t="inlineStr">
         <is>
-          <t>https://events.channelpronetwork.com/channelpro-deep-dive-the-most-profitable-cybersecurity-services-in-2027/</t>
+          <t>https://events.channelpronetwork.com/channelpro-deep-dive-perfecting-your-tool-stack/</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
@@ -3873,101 +3381,77 @@
           <t>Channel Pro Network</t>
         </is>
       </c>
-      <c r="N61" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O61" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="P61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Microsoft AI Tour - Houston</t>
+          <t>ChannelPro DEEP DIVE: The Most Profitable Cybersecurity Services in 2027</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>46540</v>
+        <v>46539</v>
       </c>
       <c r="C62" s="2" t="n"/>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>ChannelPro Network</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Texas</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>Houston</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>Host</t>
-        </is>
-      </c>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
       <c r="J62" t="inlineStr"/>
       <c r="K62" t="inlineStr"/>
       <c r="L62" s="3" t="inlineStr">
         <is>
-          <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymehouston/page/notifyme</t>
+          <t>https://events.channelpronetwork.com/channelpro-deep-dive-the-most-profitable-cybersecurity-services-in-2027/</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>Microsoft AI Tour</t>
-        </is>
-      </c>
-      <c r="N62" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O62" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="P62" t="inlineStr"/>
+          <t>Channel Pro Network</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Databricks Data+AI Summit 2027</t>
+          <t>Microsoft AI Tour - Houston</t>
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>46559</v>
-      </c>
-      <c r="C63" s="2" t="n">
-        <v>46562</v>
-      </c>
+        <v>46540</v>
+      </c>
+      <c r="C63" s="2" t="n"/>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Bay Area</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr"/>
+          <t>Texas</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3979,86 +3463,72 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" s="3" t="inlineStr">
         <is>
-          <t>https://www.databricks.com/dataaisummit/agenda</t>
+          <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymehouston/page/notifyme</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>Databricks Data+AI Summit</t>
-        </is>
-      </c>
-      <c r="N63" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O63" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="P63" t="inlineStr"/>
+          <t>Microsoft AI Tour</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ChannelPro DEEP DIVE: Where the Next Wave of MSP Revenue Is Coming From</t>
+          <t>Databricks Data+AI Summit 2027</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>46623</v>
-      </c>
-      <c r="C64" s="2" t="n"/>
+        <v>46559</v>
+      </c>
+      <c r="C64" s="2" t="n">
+        <v>46562</v>
+      </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>ChannelPro Network</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Virtual</t>
+          <t>Bay Area</t>
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Databricks</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
       <c r="J64" t="inlineStr"/>
       <c r="K64" t="inlineStr"/>
       <c r="L64" s="3" t="inlineStr">
         <is>
-          <t>https://events.channelpronetwork.com/channelpro-deep-dive-where-the-next-wave-of-msp-revenue-is-coming-from/</t>
+          <t>https://www.databricks.com/dataaisummit/agenda</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>Channel Pro Network</t>
-        </is>
-      </c>
-      <c r="N64" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O64" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="P64" t="inlineStr"/>
+          <t>Databricks Data+AI Summit</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2027 ChannelPro DEFEND: Dallas</t>
+          <t>ChannelPro DEEP DIVE: Where the Next Wave of MSP Revenue Is Coming From</t>
         </is>
       </c>
       <c r="B65" s="2" t="n">
-        <v>46644</v>
-      </c>
-      <c r="C65" s="2" t="n">
-        <v>46645</v>
-      </c>
+        <v>46623</v>
+      </c>
+      <c r="C65" s="2" t="n"/>
       <c r="D65" t="inlineStr">
         <is>
           <t>ChannelPro Network</t>
@@ -4066,18 +3536,22 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Texas</t>
+          <t>Virtual</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
       <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr"/>
       <c r="J65" t="inlineStr"/>
       <c r="K65" t="inlineStr"/>
       <c r="L65" s="3" t="inlineStr">
         <is>
-          <t>https://events.channelpronetwork.com/2027-channelpro-defend-dallas/</t>
+          <t>https://events.channelpronetwork.com/channelpro-deep-dive-where-the-next-wave-of-msp-revenue-is-coming-from/</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
@@ -4085,128 +3559,135 @@
           <t>Channel Pro Network</t>
         </is>
       </c>
-      <c r="N65" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O65" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="P65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Dreamforce 2027</t>
+          <t>2027 ChannelPro DEFEND: Dallas</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>46651</v>
+        <v>46644</v>
       </c>
       <c r="C66" s="2" t="n">
-        <v>46653</v>
+        <v>46645</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Salesforce</t>
+          <t>ChannelPro Network</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Bay Area</t>
+          <t>Texas</t>
         </is>
       </c>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>Salesforce</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>Host</t>
-        </is>
-      </c>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
       <c r="J66" t="inlineStr"/>
       <c r="K66" t="inlineStr"/>
       <c r="L66" s="3" t="inlineStr">
         <is>
-          <t>https://www.salesforce.com/dreamforce/</t>
+          <t>https://events.channelpronetwork.com/2027-channelpro-defend-dallas/</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>Dreamforce</t>
-        </is>
-      </c>
-      <c r="N66" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O66" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="P66" t="inlineStr"/>
+          <t>Channel Pro Network</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ChannelPro DEEP DIVE: The AI-Powered MSP</t>
+          <t>Dreamforce 2027</t>
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>46679</v>
-      </c>
-      <c r="C67" s="2" t="n"/>
+        <v>46651</v>
+      </c>
+      <c r="C67" s="2" t="n">
+        <v>46653</v>
+      </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>ChannelPro Network</t>
+          <t>Salesforce</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Virtual</t>
+          <t>Bay Area</t>
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr"/>
-      <c r="I67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Salesforce</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
       <c r="J67" t="inlineStr"/>
       <c r="K67" t="inlineStr"/>
       <c r="L67" s="3" t="inlineStr">
         <is>
+          <t>https://www.salesforce.com/dreamforce/</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>Dreamforce</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>ChannelPro DEEP DIVE: The AI-Powered MSP</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="n">
+        <v>46679</v>
+      </c>
+      <c r="C68" s="2" t="n"/>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>ChannelPro Network</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" s="3" t="inlineStr">
+        <is>
           <t>https://events.channelpronetwork.com/channelpro-deep-dive-the-ai-powered-msp/</t>
         </is>
       </c>
-      <c r="M67" t="inlineStr">
+      <c r="M68" t="inlineStr">
         <is>
           <t>Channel Pro Network</t>
         </is>
       </c>
-      <c r="N67" s="2" t="n">
-        <v>46322</v>
-      </c>
-      <c r="O67" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="P67" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="O2:O5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"New,Attending,Skip"</formula1>
-    </dataValidation>
-  </dataValidations>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -4242,7 +3723,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L49" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L50" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L51" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L53" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L52" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L54" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L55" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L56" r:id="rId38"/>
@@ -4257,10 +3738,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L65" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L66" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L67" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L68" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId50"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId51"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Partnership Leaders, CMA, CRN/Channel Co sources; trusted channel sources, borrowed flagship cities
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TLMW817qEmLPfhM4KiByCq
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -146,8 +146,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Events" displayName="Events" ref="A1:M68" headerRowCount="1">
-  <autoFilter ref="A1:M68"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Events" displayName="Events" ref="A1:M71" headerRowCount="1">
+  <autoFilter ref="A1:M71"/>
   <tableColumns count="13">
     <tableColumn id="1" name="Name"/>
     <tableColumn id="2" name="Date"/>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M68"/>
+  <dimension ref="A1:M71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2939,16 +2939,16 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Cloudflare Immerse</t>
+          <t>Catalyst Breakfast at Microsoft Ignite</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>46346</v>
+        <v>46344</v>
       </c>
       <c r="C52" s="2" t="n"/>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Cloudflare</t>
+          <t>Partnership Leaders</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2958,7 +2958,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Bay Area</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2968,43 +2968,46 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Cloudflare</t>
-        </is>
-      </c>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
       <c r="L52" s="3" t="inlineStr">
         <is>
-          <t>https://fieldmarketing.www.cloudflare.com/cloudflareimmersebayarea?_gl=1*1ge1j1x*_gcl_au*MjMxOTM0MjE4LjE3NTkzNjYwMjI.*_ga*ZmI3OTU3NjUtZDkyOC00M2I3LWJiOGYtNzQ5ZjJlZGUxYWFm*_ga_SQCRB0TXZW*czE3NjU0NjEwMDIkbzMkZzEkdDE3NjU0NjEwNTkkajMkbDAkaDAkZHVGb1hkWDJpQmU2OUExYjJSSl92c2xTbkxWQURDZTlUSWc.</t>
+          <t>https://www.joincatalyst.com/catalyst-breakfast-at-microsoft-ignite</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>Legacy tracker 2026</t>
+          <t>Partnership Leaders events</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Gartner / Evanta Seattle CIO Community Executive Summit</t>
+          <t>Cloudflare Immerse</t>
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>46357</v>
+        <v>46346</v>
       </c>
       <c r="C53" s="2" t="n"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Google Cloud / Cloudflare / Dynatrace</t>
+          <t>Cloudflare</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Bay Area</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Bay Area</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3014,12 +3017,12 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Google, Dynatrace, Cloudflare</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>Invite/application-based; no public attendee fee</t>
+          <t>Cloudflare</t>
+        </is>
+      </c>
+      <c r="L53" s="3" t="inlineStr">
+        <is>
+          <t>https://fieldmarketing.www.cloudflare.com/cloudflareimmersebayarea?_gl=1*1ge1j1x*_gcl_au*MjMxOTM0MjE4LjE3NTkzNjYwMjI.*_ga*ZmI3OTU3NjUtZDkyOC00M2I3LWJiOGYtNzQ5ZjJlZGUxYWFm*_ga_SQCRB0TXZW*czE3NjU0NjEwMDIkbzMkZzEkdDE3NjU0NjEwNTkkajMkbDAkaDAkZHVGb1hkWDJpQmU2OUExYjJSSl92c2xTbkxWQURDZTlUSWc.</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -3031,146 +3034,135 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>MSP Summit: AI Symposium</t>
+          <t>Gartner / Evanta Seattle CIO Community Executive Summit</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>46365</v>
+        <v>46357</v>
       </c>
       <c r="C54" s="2" t="n"/>
-      <c r="D54" t="inlineStr"/>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Google Cloud / Cloudflare / Dynatrace</t>
+        </is>
+      </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>New York</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
+          <t>Seattle</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Seattle</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" s="3" t="inlineStr">
-        <is>
-          <t>https://themspsummit.com/msp-summit-ai-symposium/</t>
+          <t>Google, Dynatrace, Cloudflare</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Invite/application-based; no public attendee fee</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>MSP Summit / events calendar</t>
+          <t>Legacy tracker 2026</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Microsoft AI Tour - Seattle</t>
+          <t>CMA Power Circles</t>
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>46365</v>
+        <v>46358</v>
       </c>
       <c r="C55" s="2" t="n"/>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Channel Marketing Association</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Seattle</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>Seattle</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>Host</t>
-        </is>
-      </c>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr"/>
       <c r="L55" s="3" t="inlineStr">
         <is>
-          <t>https://aitour.microsoft.com/flow/microsoft/seattle27/citylanding/page/cityhome</t>
+          <t>https://www.channelmarketingassociation.com/industry-events</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>Microsoft AI Tour</t>
+          <t>Channel Marketing Association events</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Microsoft AI Tour - Mumbai</t>
+          <t>MSP Summit: AI Symposium</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>46428</v>
+        <v>46365</v>
       </c>
       <c r="C56" s="2" t="n"/>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
+      <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
-          <t>India</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>Mumbai</t>
-        </is>
-      </c>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>Host</t>
-        </is>
-      </c>
+      <c r="I56" t="inlineStr"/>
       <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr"/>
       <c r="L56" s="3" t="inlineStr">
         <is>
-          <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymemumbai/page/notifyme</t>
+          <t>https://themspsummit.com/msp-summit-ai-symposium/</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>Microsoft AI Tour</t>
+          <t>MSP Summit / events calendar</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Microsoft AI Tour - Bengaluru</t>
+          <t>Microsoft AI Tour - Seattle</t>
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>46433</v>
+        <v>46365</v>
       </c>
       <c r="C57" s="2" t="n"/>
       <c r="D57" t="inlineStr">
@@ -3180,12 +3172,12 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="G57" t="inlineStr"/>
@@ -3203,7 +3195,7 @@
       <c r="K57" t="inlineStr"/>
       <c r="L57" s="3" t="inlineStr">
         <is>
-          <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymebengaluru/page/notifyme</t>
+          <t>https://aitour.microsoft.com/flow/microsoft/seattle27/citylanding/page/cityhome</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
@@ -3215,318 +3207,318 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ChannelPro DEEP DIVE: Cybersecurity in the Age of AI</t>
+          <t>Microsoft AI Tour - Mumbai</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>46434</v>
+        <v>46428</v>
       </c>
       <c r="C58" s="2" t="n"/>
       <c r="D58" t="inlineStr">
         <is>
-          <t>ChannelPro Network</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
       <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr"/>
       <c r="L58" s="3" t="inlineStr">
         <is>
-          <t>https://events.channelpronetwork.com/channelpro-deep-dive-cybersecurity-in-the-age-of-ai/</t>
+          <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymemumbai/page/notifyme</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>Channel Pro Network</t>
+          <t>Microsoft AI Tour</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Xchange 2027</t>
+          <t>Microsoft AI Tour - Bengaluru</t>
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>46453</v>
-      </c>
-      <c r="C59" s="2" t="n">
-        <v>46455</v>
-      </c>
+        <v>46433</v>
+      </c>
+      <c r="C59" s="2" t="n"/>
       <c r="D59" t="inlineStr">
         <is>
-          <t>The Channel Company</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Texas</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr"/>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
       <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
       <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr"/>
       <c r="L59" s="3" t="inlineStr">
         <is>
-          <t>https://event.thechannelco.com/xchange-march/</t>
+          <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymebengaluru/page/notifyme</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>Xchange (The Channel Co)</t>
+          <t>Microsoft AI Tour</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Microsoft AI Tour - New York City</t>
+          <t>ChannelPro DEEP DIVE: Cybersecurity in the Age of AI</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>46464</v>
+        <v>46434</v>
       </c>
       <c r="C60" s="2" t="n"/>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>ChannelPro Network</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>New York</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>New York City</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>Host</t>
-        </is>
-      </c>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
       <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr"/>
       <c r="L60" s="3" t="inlineStr">
         <is>
-          <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymenyc/page/notifyme</t>
+          <t>https://events.channelpronetwork.com/channelpro-deep-dive-cybersecurity-in-the-age-of-ai/</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>Microsoft AI Tour</t>
+          <t>Channel Pro Network</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ChannelPro DEEP DIVE: Perfecting Your Tool Stack</t>
+          <t>Xchange 2027</t>
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>46483</v>
-      </c>
-      <c r="C61" s="2" t="n"/>
+        <v>46453</v>
+      </c>
+      <c r="C61" s="2" t="n">
+        <v>46455</v>
+      </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>ChannelPro Network</t>
+          <t>The Channel Company</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Virtual</t>
+          <t>Texas</t>
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
+      <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr"/>
       <c r="K61" t="inlineStr"/>
       <c r="L61" s="3" t="inlineStr">
         <is>
-          <t>https://events.channelpronetwork.com/channelpro-deep-dive-perfecting-your-tool-stack/</t>
+          <t>https://event.thechannelco.com/xchange-march/</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>Channel Pro Network</t>
+          <t>Xchange (The Channel Co)</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ChannelPro DEEP DIVE: The Most Profitable Cybersecurity Services in 2027</t>
+          <t>Microsoft AI Tour - New York City</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>46539</v>
+        <v>46464</v>
       </c>
       <c r="C62" s="2" t="n"/>
       <c r="D62" t="inlineStr">
         <is>
-          <t>ChannelPro Network</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
       <c r="J62" t="inlineStr"/>
       <c r="K62" t="inlineStr"/>
       <c r="L62" s="3" t="inlineStr">
         <is>
-          <t>https://events.channelpronetwork.com/channelpro-deep-dive-the-most-profitable-cybersecurity-services-in-2027/</t>
+          <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymenyc/page/notifyme</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>Channel Pro Network</t>
+          <t>Microsoft AI Tour</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Microsoft AI Tour - Houston</t>
+          <t>ChannelPro DEEP DIVE: Perfecting Your Tool Stack</t>
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>46540</v>
+        <v>46483</v>
       </c>
       <c r="C63" s="2" t="n"/>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>ChannelPro Network</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Texas</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>Houston</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>Host</t>
-        </is>
-      </c>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr"/>
       <c r="K63" t="inlineStr"/>
       <c r="L63" s="3" t="inlineStr">
         <is>
-          <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymehouston/page/notifyme</t>
+          <t>https://events.channelpronetwork.com/channelpro-deep-dive-perfecting-your-tool-stack/</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>Microsoft AI Tour</t>
+          <t>Channel Pro Network</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Databricks Data+AI Summit 2027</t>
+          <t>Global Channel Growth Summit 2027</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>46559</v>
+        <v>46490</v>
       </c>
       <c r="C64" s="2" t="n">
-        <v>46562</v>
+        <v>46492</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Databricks</t>
+          <t>Channel Marketing Association</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Bay Area</t>
+          <t>Texas</t>
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>Databricks</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>Host</t>
-        </is>
-      </c>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
       <c r="J64" t="inlineStr"/>
       <c r="K64" t="inlineStr"/>
       <c r="L64" s="3" t="inlineStr">
         <is>
-          <t>https://www.databricks.com/dataaisummit/agenda</t>
+          <t>https://www.channelmarketingassociation.com/Global-Summit-2027</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>Databricks Data+AI Summit</t>
+          <t>CMA Global Channel Growth Summit</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ChannelPro DEEP DIVE: Where the Next Wave of MSP Revenue Is Coming From</t>
+          <t>ChannelPro DEEP DIVE: The Most Profitable Cybersecurity Services in 2027</t>
         </is>
       </c>
       <c r="B65" s="2" t="n">
-        <v>46623</v>
+        <v>46539</v>
       </c>
       <c r="C65" s="2" t="n"/>
       <c r="D65" t="inlineStr">
@@ -3551,7 +3543,7 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" s="3" t="inlineStr">
         <is>
-          <t>https://events.channelpronetwork.com/channelpro-deep-dive-where-the-next-wave-of-msp-revenue-is-coming-from/</t>
+          <t>https://events.channelpronetwork.com/channelpro-deep-dive-the-most-profitable-cybersecurity-services-in-2027/</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
@@ -3563,18 +3555,16 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2027 ChannelPro DEFEND: Dallas</t>
+          <t>Microsoft AI Tour - Houston</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>46644</v>
-      </c>
-      <c r="C66" s="2" t="n">
-        <v>46645</v>
-      </c>
+        <v>46540</v>
+      </c>
+      <c r="C66" s="2" t="n"/>
       <c r="D66" t="inlineStr">
         <is>
-          <t>ChannelPro Network</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3582,38 +3572,50 @@
           <t>Texas</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
       <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
       <c r="J66" t="inlineStr"/>
       <c r="K66" t="inlineStr"/>
       <c r="L66" s="3" t="inlineStr">
         <is>
-          <t>https://events.channelpronetwork.com/2027-channelpro-defend-dallas/</t>
+          <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymehouston/page/notifyme</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>Channel Pro Network</t>
+          <t>Microsoft AI Tour</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Dreamforce 2027</t>
+          <t>Databricks Data+AI Summit 2027</t>
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>46651</v>
+        <v>46559</v>
       </c>
       <c r="C67" s="2" t="n">
-        <v>46653</v>
+        <v>46562</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Salesforce</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3625,7 +3627,7 @@
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Salesforce</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3637,23 +3639,23 @@
       <c r="K67" t="inlineStr"/>
       <c r="L67" s="3" t="inlineStr">
         <is>
-          <t>https://www.salesforce.com/dreamforce/</t>
+          <t>https://www.databricks.com/dataaisummit/agenda</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>Dreamforce</t>
+          <t>Databricks Data+AI Summit</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ChannelPro DEEP DIVE: The AI-Powered MSP</t>
+          <t>ChannelPro DEEP DIVE: Where the Next Wave of MSP Revenue Is Coming From</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>46679</v>
+        <v>46623</v>
       </c>
       <c r="C68" s="2" t="n"/>
       <c r="D68" t="inlineStr">
@@ -3678,10 +3680,141 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" s="3" t="inlineStr">
         <is>
+          <t>https://events.channelpronetwork.com/channelpro-deep-dive-where-the-next-wave-of-msp-revenue-is-coming-from/</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>Channel Pro Network</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2027 ChannelPro DEFEND: Dallas</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="n">
+        <v>46644</v>
+      </c>
+      <c r="C69" s="2" t="n">
+        <v>46645</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>ChannelPro Network</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Texas</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" s="3" t="inlineStr">
+        <is>
+          <t>https://events.channelpronetwork.com/2027-channelpro-defend-dallas/</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>Channel Pro Network</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Dreamforce 2027</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="n">
+        <v>46651</v>
+      </c>
+      <c r="C70" s="2" t="n">
+        <v>46653</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Salesforce</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Bay Area</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Salesforce</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" s="3" t="inlineStr">
+        <is>
+          <t>https://www.salesforce.com/dreamforce/</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>Dreamforce</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>ChannelPro DEEP DIVE: The AI-Powered MSP</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="n">
+        <v>46679</v>
+      </c>
+      <c r="C71" s="2" t="n"/>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>ChannelPro Network</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" s="3" t="inlineStr">
+        <is>
           <t>https://events.channelpronetwork.com/channelpro-deep-dive-the-ai-powered-msp/</t>
         </is>
       </c>
-      <c r="M68" t="inlineStr">
+      <c r="M71" t="inlineStr">
         <is>
           <t>Channel Pro Network</t>
         </is>
@@ -3724,7 +3857,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L50" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L51" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L52" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L54" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L53" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L55" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L56" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L57" r:id="rId39"/>
@@ -3739,10 +3872,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L66" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L67" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L68" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L69" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L70" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L71" r:id="rId53"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId51"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId54"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CSV dates as plain readable text (one Date column) so Excel has nothing to convert
Also tidy legacy import host handling for 'A / B' account labels.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TLMW817qEmLPfhM4KiByCq
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="2026" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2027" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2027" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -147,8 +147,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Events2026" displayName="Events2026" ref="A1:M36" headerRowCount="1">
-  <autoFilter ref="A1:M36"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Events2026" displayName="Events2026" ref="A1:M34" headerRowCount="1">
+  <autoFilter ref="A1:M34"/>
   <tableColumns count="13">
     <tableColumn id="1" name="Name"/>
     <tableColumn id="2" name="Date"/>
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -615,16 +615,16 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AI Agents Seattle – August 2026</t>
+          <t>AI Agents in the Wild: Building, Scaling &amp; Deploying in Production</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="C3" s="2" t="n"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>AI / Claude ecosystem</t>
+          <t>Salesforce</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Bellevue</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -644,7 +644,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>AWS, Salesforce</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -661,16 +661,16 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AI Agents in the Wild: Building, Scaling &amp; Deploying in Production</t>
+          <t>NVIDIA Spark Hack: Seattle</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>46246</v>
+        <v>46248</v>
       </c>
       <c r="C4" s="2" t="n"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Salesforce / AWS</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Bellevue</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -690,12 +690,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>AWS, Salesforce</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Not publicly listed</t>
+          <t>No public fee listed; approval required</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -707,16 +707,16 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NVIDIA Spark Hack: Seattle</t>
+          <t>ISV Partner Event</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>46248</v>
+        <v>46254</v>
       </c>
       <c r="C5" s="2" t="n"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>ServiceNow</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -736,12 +736,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>ServiceNow</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>No public fee listed; approval required</t>
+          <t>Free</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -753,16 +753,18 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ISV Partner Event</t>
+          <t>MICROSOFT 365, DATA &amp; POWER PLATFORM CONFERENCES</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>46254</v>
-      </c>
-      <c r="C6" s="2" t="n"/>
+        <v>46258</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>46262</v>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ServiceNow</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -782,12 +784,17 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>ServiceNow</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Free</t>
+          <t>1595-2695</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.techcon365.com/Seattle/</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -799,7 +806,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MICROSOFT 365, DATA &amp; POWER PLATFORM CONFERENCES</t>
+          <t>TechCon 365, DATACON &amp; PWRCON Seattle 2026</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
@@ -835,12 +842,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>1595-2695</t>
-        </is>
-      </c>
-      <c r="L7" s="3" t="inlineStr">
-        <is>
-          <t>https://www.techcon365.com/Seattle/</t>
+          <t>$1,825–$2,995 currently, depending on pass</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -852,18 +854,18 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TechCon 365, DATACON &amp; PWRCON Seattle 2026</t>
+          <t>AWS Marketplace Seller Forum</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>46258</v>
+        <v>46266</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>46262</v>
+        <v>46267</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -873,7 +875,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Bellevue</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -883,12 +885,17 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>$1,825–$2,995 currently, depending on pass</t>
+          <t>Invite only event</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>https://aws.amazon.com/marketplace/resources/events/seller-conference</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -900,18 +907,16 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AWS Marketplace Seller Forum</t>
+          <t>AI, Zero Trust &amp; Enterprise Resilience in the Age of Continuous Disruption</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>46266</v>
-      </c>
-      <c r="C9" s="2" t="n">
-        <v>46267</v>
-      </c>
+        <v>46275</v>
+      </c>
+      <c r="C9" s="2" t="n"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Intuit</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -931,17 +936,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Oracle, Intuit</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Invite only event</t>
-        </is>
-      </c>
-      <c r="L9" s="3" t="inlineStr">
-        <is>
-          <t>https://aws.amazon.com/marketplace/resources/events/seller-conference</t>
+          <t>Not publicly listed</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -953,7 +953,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AI, Zero Trust &amp; Enterprise Resilience in the Age of Continuous Disruption</t>
+          <t>CISOMeet Seattle</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -962,7 +962,7 @@
       <c r="C10" s="2" t="n"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Intuit / Oracle</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -982,12 +982,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Oracle, Intuit</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Not publicly listed</t>
+          <t>No public fee listed; CISO/Sr. InfoSec qualification</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -999,7 +999,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CISOMeet Seattle</t>
+          <t>World Forum</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
@@ -1008,17 +1008,17 @@
       <c r="C11" s="2" t="n"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>ServiceNow</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Bellevue</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1028,12 +1028,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>SAP</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>No public fee listed; CISO/Sr. InfoSec qualification</t>
+          <t>ServiceNow</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.servicenow.com/events/world-forum.html</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1045,26 +1045,28 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>World Forum</t>
+          <t>Dreamforce 2026</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>46275</v>
-      </c>
-      <c r="C12" s="2" t="n"/>
+        <v>46280</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>46282</v>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ServiceNow</t>
+          <t>Salesforce</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Bay Area</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1074,12 +1076,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>ServiceNow</t>
+          <t>Salesforce</t>
         </is>
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>https://www.servicenow.com/events/world-forum.html</t>
+          <t>https://www.salesforce.com/dreamforce/?d=pb</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1091,28 +1093,28 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Dreamforce 2026</t>
+          <t>Amazon Accelerate 2026</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46280</v>
+        <v>46287</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>46282</v>
+        <v>46289</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Salesforce</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Bay Area</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1122,12 +1124,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Salesforce</t>
-        </is>
-      </c>
-      <c r="L13" s="3" t="inlineStr">
-        <is>
-          <t>https://www.salesforce.com/dreamforce/?d=pb</t>
+          <t>AWS</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Price not publicly surfaced; $100 early-bird discount through Aug 8</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1139,18 +1141,16 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Amazon Accelerate 2026</t>
+          <t>Build with Gemini – Seattle</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>46287</v>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>46289</v>
-      </c>
+        <v>46295</v>
+      </c>
+      <c r="C14" s="2" t="n"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Amazon / AWS ecosystem</t>
+          <t>Google Cloud</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1170,12 +1170,12 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Price not publicly surfaced; $100 early-bird discount through Aug 8</t>
+          <t>Free / complimentary</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1187,18 +1187,16 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>IA40 Summit 2026</t>
+          <t>Official Cybersecurity Summit – Seattle/Bellevue</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>46294</v>
-      </c>
-      <c r="C15" s="2" t="n">
-        <v>46295</v>
-      </c>
+        <v>46296</v>
+      </c>
+      <c r="C15" s="2" t="n"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>AI ecosystem / Microsoft / AWS / Databricks</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1208,7 +1206,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Bellevue</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1218,12 +1216,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Microsoft, AWS, Databricks</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Invite-only / no public fee</t>
+          <t>$250 standard admission</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1235,26 +1233,23 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Build with Gemini – Seattle</t>
+          <t>Cypher 2026</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>46295</v>
-      </c>
-      <c r="C16" s="2" t="n"/>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Google Cloud</t>
-        </is>
+        <v>46301</v>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>46303</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1262,14 +1257,14 @@
           <t>In-person</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
-      </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Free / complimentary</t>
+          <t>7000 (INR)</t>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>https://kripeshadwani.com/best-tech-events-in-india/#ai-impact-summit-2026</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1281,26 +1276,26 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Official Cybersecurity Summit – Seattle/Bellevue</t>
+          <t>World Forum</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>46296</v>
+        <v>46301</v>
       </c>
       <c r="C17" s="2" t="n"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>IBM / Cybersecurity ecosystem</t>
+          <t>ServiceNow</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Bellevue</t>
+          <t>Mumbai</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1310,12 +1305,12 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>IBM</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>$250 standard admission</t>
+          <t>ServiceNow</t>
+        </is>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.servicenow.com/events/world-forum.html</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1327,23 +1322,23 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Cypher 2026</t>
+          <t>TechCrunch Disrupt 2026</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>46301</v>
+        <v>46308</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>46303</v>
+        <v>46310</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bay Area</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1353,12 +1348,12 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>7000 (INR)</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>https://kripeshadwani.com/best-tech-events-in-india/#ai-impact-summit-2026</t>
+          <t>https://techcrunch.com/events/tc-disrupt-2026/</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1370,26 +1365,26 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>World Forum</t>
+          <t>ElevateIT Seattle Technology Summit 2026</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="C19" s="2" t="n"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>ServiceNow</t>
+          <t>Nutanix</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Mumbai</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1399,12 +1394,12 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>ServiceNow</t>
-        </is>
-      </c>
-      <c r="L19" s="3" t="inlineStr">
-        <is>
-          <t>https://www.servicenow.com/events/world-forum.html</t>
+          <t>Nutanix</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Not publicly listed</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1416,14 +1411,19 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TechCrunch Disrupt 2026</t>
+          <t>Cloudflare Connect</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>46308</v>
+        <v>46314</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>46310</v>
+        <v>46317</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Cloudflare</t>
+        </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1440,14 +1440,14 @@
           <t>In-person</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>Not mentioned</t>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Cloudflare</t>
         </is>
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>https://techcrunch.com/events/tc-disrupt-2026/</t>
+          <t>https://www.cloudflare.com/en-gb/lp/cloudflare-connect-2026/</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1459,16 +1459,18 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ElevateIT Seattle Technology Summit 2026</t>
+          <t>Seattle AI Week 2026</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>46309</v>
-      </c>
-      <c r="C21" s="2" t="n"/>
+        <v>46321</v>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>46325</v>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Nutanix / Enterprise IT ecosystem</t>
+          <t>Multi-vendor</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1486,14 +1488,9 @@
           <t>In-person</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Nutanix</t>
-        </is>
-      </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Not publicly listed</t>
+          <t>Varies by event; flagship Summit EB $175</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1505,28 +1502,28 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Cloudflare Connect</t>
+          <t>Agents in NYC</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>46314</v>
+        <v>46323</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>46317</v>
+        <v>46323</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Cloudflare</t>
+          <t>Datadog, Albert Zhao, Datadog</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Bay Area</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1536,35 +1533,42 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Cloudflare</t>
-        </is>
-      </c>
+          <t>Datadog</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>https://www.cloudflare.com/en-gb/lp/cloudflare-connect-2026/</t>
+          <t>https://luma.com/agentsinnyc</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Legacy tracker 2026</t>
+          <t>Luma NYC</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Seattle AI Week 2026</t>
+          <t>SecureWorld Seattle 2026</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>46321</v>
+        <v>46330</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>46325</v>
+        <v>46331</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Multi-vendor / AI ecosystem</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1574,7 +1578,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Bellevue</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1582,9 +1586,14 @@
           <t>In-person</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Google, Cohesity, Blue Yonder, OpenAI</t>
+        </is>
+      </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Varies by event; flagship Summit EB $175</t>
+          <t>Multiple pass types; current price not publicly surfaced in indexed page</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -1596,28 +1605,28 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Agents in NYC</t>
+          <t>PASS Data Community Summit West</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>46323</v>
+        <v>46335</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>46323</v>
+        <v>46337</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Datadog, Albert Zhao, Datadog</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1625,44 +1634,30 @@
           <t>In-person</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Datadog</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>Host</t>
-        </is>
-      </c>
-      <c r="L24" s="3" t="inlineStr">
-        <is>
-          <t>https://luma.com/agentsinnyc</t>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>$1,790–$1,990 for published 2-day ticket</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Luma NYC</t>
+          <t>Legacy tracker 2026</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SecureWorld Seattle 2026</t>
+          <t>SaaSify Partner Central Agentic Workshop</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>46330</v>
+        <v>46338</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>46331</v>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>OpenAI / Google Cloud / Cohesity / Blue Yonder</t>
-        </is>
-      </c>
+        <v>46338</v>
+      </c>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>Seattle</t>
@@ -1670,7 +1665,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Bellevue</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1680,35 +1675,36 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Google, Cohesity, Blue Yonder, OpenAI</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>Multiple pass types; current price not publicly surfaced in indexed page</t>
+          <t>AWS</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/saasify-partner-central-agentic-workshop-tickets-2003698327636</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Legacy tracker 2026</t>
+          <t>Eventbrite Seattle - AWS/Microsoft/Google</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PASS Data Community Summit West</t>
+          <t>Identity, AI &amp; Cybersecurity: Securing the Enterprise in an Agentic World</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>46335</v>
-      </c>
-      <c r="C26" s="2" t="n">
-        <v>46337</v>
-      </c>
+        <v>46339</v>
+      </c>
+      <c r="C26" s="2" t="n"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Data / Cloud ecosystem</t>
+          <t>Seattle Data, AI &amp; Security</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1718,7 +1714,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Bellevue</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1726,37 +1722,54 @@
           <t>In-person</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>$1,790–$1,990 for published 2-day ticket</t>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Seattle Data, AI &amp; Security</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" s="3" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/seattledataaiandsecurity/events/316481475/</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Legacy tracker 2026</t>
+          <t>Meetup Seattle - AWS</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SaaSify Partner Central Agentic Workshop</t>
+          <t>Microsoft Ignite 2026</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>46338</v>
+        <v>46343</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>46338</v>
+        <v>46346</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Bay Area</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1766,43 +1779,41 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="L27" s="3" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/saasify-partner-central-agentic-workshop-tickets-2003698327636</t>
+          <t>https://ignite.microsoft.com/en-US/home</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Eventbrite Seattle - AWS/Microsoft/Google</t>
+          <t>Legacy tracker 2026</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Identity, AI &amp; Cybersecurity: Securing the Enterprise in an Agentic World</t>
+          <t>SaaSify Partner Central Agentic Workshop</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>46339</v>
-      </c>
-      <c r="C28" s="2" t="n"/>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Seattle Data, AI &amp; Security</t>
-        </is>
-      </c>
+        <v>46343</v>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>46343</v>
+      </c>
+      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Bay Area</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Bellevue</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1812,84 +1823,86 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>Seattle Data, AI &amp; Security</t>
-        </is>
-      </c>
+          <t>AWS</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/seattledataaiandsecurity/events/316481475/</t>
+          <t>https://www.eventbrite.com/e/saasify-partner-central-agentic-workshop-tickets-2003695905391</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Meetup Seattle - AWS</t>
+          <t>Eventbrite SF - cloud partner</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Microsoft Ignite 2026</t>
+          <t>Catalyst Breakfast at Microsoft Ignite</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>46343</v>
-      </c>
-      <c r="C29" s="2" t="n">
-        <v>46346</v>
-      </c>
+        <v>46344</v>
+      </c>
+      <c r="C29" s="2" t="n"/>
       <c r="D29" t="inlineStr">
         <is>
+          <t>Partnership Leaders</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Bay Area</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Bay Area</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>San Francisco</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>In-person</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
       <c r="L29" s="3" t="inlineStr">
         <is>
-          <t>https://ignite.microsoft.com/en-US/home</t>
+          <t>https://www.joincatalyst.com/catalyst-breakfast-at-microsoft-ignite</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Legacy tracker 2026</t>
+          <t>Partnership Leaders events</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SaaSify Partner Central Agentic Workshop</t>
+          <t>Cloudflare Immerse</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>46343</v>
-      </c>
-      <c r="C30" s="2" t="n">
-        <v>46343</v>
+        <v>46346</v>
+      </c>
+      <c r="C30" s="2" t="n"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Cloudflare</t>
+        </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1898,7 +1911,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>Bay Area</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1908,43 +1921,43 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Cloudflare</t>
         </is>
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/saasify-partner-central-agentic-workshop-tickets-2003695905391</t>
+          <t>https://fieldmarketing.www.cloudflare.com/cloudflareimmersebayarea?_gl=1*1ge1j1x*_gcl_au*MjMxOTM0MjE4LjE3NTkzNjYwMjI.*_ga*ZmI3OTU3NjUtZDkyOC00M2I3LWJiOGYtNzQ5ZjJlZGUxYWFm*_ga_SQCRB0TXZW*czE3NjU0NjEwMDIkbzMkZzEkdDE3NjU0NjEwNTkkajMkbDAkaDAkZHVGb1hkWDJpQmU2OUExYjJSSl92c2xTbkxWQURDZTlUSWc.</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Eventbrite SF - cloud partner</t>
+          <t>Legacy tracker 2026</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Catalyst Breakfast at Microsoft Ignite</t>
+          <t>Gartner / Evanta Seattle CIO Community Executive Summit</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>46344</v>
+        <v>46357</v>
       </c>
       <c r="C31" s="2" t="n"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Partnership Leaders</t>
+          <t>Google Cloud</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Bay Area</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1954,220 +1967,142 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="L31" s="3" t="inlineStr">
-        <is>
-          <t>https://www.joincatalyst.com/catalyst-breakfast-at-microsoft-ignite</t>
+          <t>Google, Dynatrace, Cloudflare</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Invite/application-based; no public attendee fee</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>Partnership Leaders events</t>
+          <t>Legacy tracker 2026</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Cloudflare Immerse</t>
+          <t>CMA Power Circles</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>46346</v>
+        <v>46358</v>
       </c>
       <c r="C32" s="2" t="n"/>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Cloudflare</t>
+          <t>Channel Marketing Association</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Bay Area</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Bay Area</t>
-        </is>
-      </c>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>In-person</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>Cloudflare</t>
-        </is>
-      </c>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
       <c r="L32" s="3" t="inlineStr">
         <is>
-          <t>https://fieldmarketing.www.cloudflare.com/cloudflareimmersebayarea?_gl=1*1ge1j1x*_gcl_au*MjMxOTM0MjE4LjE3NTkzNjYwMjI.*_ga*ZmI3OTU3NjUtZDkyOC00M2I3LWJiOGYtNzQ5ZjJlZGUxYWFm*_ga_SQCRB0TXZW*czE3NjU0NjEwMDIkbzMkZzEkdDE3NjU0NjEwNTkkajMkbDAkaDAkZHVGb1hkWDJpQmU2OUExYjJSSl92c2xTbkxWQURDZTlUSWc.</t>
+          <t>https://www.channelmarketingassociation.com/industry-events</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Legacy tracker 2026</t>
+          <t>Channel Marketing Association events</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Gartner / Evanta Seattle CIO Community Executive Summit</t>
+          <t>MSP Summit: AI Symposium</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>46357</v>
+        <v>46365</v>
       </c>
       <c r="C33" s="2" t="n"/>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Google Cloud / Cloudflare / Dynatrace</t>
-        </is>
-      </c>
+      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Seattle</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Seattle</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>In-person</t>
-        </is>
-      </c>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Google, Dynatrace, Cloudflare</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>Invite/application-based; no public attendee fee</t>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" s="3" t="inlineStr">
+        <is>
+          <t>https://themspsummit.com/msp-summit-ai-symposium/</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Legacy tracker 2026</t>
+          <t>MSP Summit / events calendar</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CMA Power Circles</t>
+          <t>Microsoft AI Tour - Seattle</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>46358</v>
+        <v>46365</v>
       </c>
       <c r="C34" s="2" t="n"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Channel Marketing Association</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
+          <t>Seattle</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Seattle</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
       <c r="L34" s="3" t="inlineStr">
         <is>
-          <t>https://www.channelmarketingassociation.com/industry-events</t>
+          <t>https://aitour.microsoft.com/flow/microsoft/seattle27/citylanding/page/cityhome</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
-        <is>
-          <t>Channel Marketing Association events</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>MSP Summit: AI Symposium</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="n">
-        <v>46365</v>
-      </c>
-      <c r="C35" s="2" t="n"/>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>New York</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="L35" s="3" t="inlineStr">
-        <is>
-          <t>https://themspsummit.com/msp-summit-ai-symposium/</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>MSP Summit / events calendar</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Microsoft AI Tour - Seattle</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="n">
-        <v>46365</v>
-      </c>
-      <c r="C36" s="2" t="n"/>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Seattle</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>Seattle</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>Host</t>
-        </is>
-      </c>
-      <c r="L36" s="3" t="inlineStr">
-        <is>
-          <t>https://aitour.microsoft.com/flow/microsoft/seattle27/citylanding/page/cityhome</t>
-        </is>
-      </c>
-      <c r="M36" t="inlineStr">
         <is>
           <t>Microsoft AI Tour</t>
         </is>
@@ -2175,24 +2110,24 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -2317,6 +2252,7 @@
           <t>Mumbai</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -2327,6 +2263,8 @@
           <t>Host</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymemumbai/page/notifyme</t>
@@ -2363,6 +2301,7 @@
           <t>Bengaluru</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -2373,6 +2312,8 @@
           <t>Host</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymebengaluru/page/notifyme</t>
@@ -2404,11 +2345,16 @@
           <t>Virtual</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>Virtual</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" s="3" t="inlineStr">
         <is>
           <t>https://events.channelpronetwork.com/channelpro-deep-dive-cybersecurity-in-the-age-of-ai/</t>
@@ -2442,6 +2388,12 @@
           <t>Texas</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" s="3" t="inlineStr">
         <is>
           <t>https://event.thechannelco.com/xchange-march/</t>
@@ -2478,6 +2430,7 @@
           <t>New York City</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -2488,6 +2441,8 @@
           <t>Host</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymenyc/page/notifyme</t>
@@ -2519,11 +2474,16 @@
           <t>Virtual</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>Virtual</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" s="3" t="inlineStr">
         <is>
           <t>https://events.channelpronetwork.com/channelpro-deep-dive-perfecting-your-tool-stack/</t>
@@ -2557,6 +2517,12 @@
           <t>Texas</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" s="3" t="inlineStr">
         <is>
           <t>https://www.channelmarketingassociation.com/Global-Summit-2027</t>
@@ -2588,11 +2554,16 @@
           <t>Virtual</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>Virtual</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" s="3" t="inlineStr">
         <is>
           <t>https://events.channelpronetwork.com/channelpro-deep-dive-the-most-profitable-cybersecurity-services-in-2027/</t>
@@ -2629,6 +2600,7 @@
           <t>Houston</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -2639,6 +2611,8 @@
           <t>Host</t>
         </is>
       </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymehouston/page/notifyme</t>
@@ -2672,6 +2646,8 @@
           <t>Bay Area</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>Databricks</t>
@@ -2682,6 +2658,8 @@
           <t>Host</t>
         </is>
       </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" s="3" t="inlineStr">
         <is>
           <t>https://www.databricks.com/dataaisummit/agenda</t>
@@ -2713,11 +2691,16 @@
           <t>Virtual</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>Virtual</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
       <c r="L12" s="3" t="inlineStr">
         <is>
           <t>https://events.channelpronetwork.com/channelpro-deep-dive-where-the-next-wave-of-msp-revenue-is-coming-from/</t>
@@ -2751,6 +2734,12 @@
           <t>Texas</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" s="3" t="inlineStr">
         <is>
           <t>https://events.channelpronetwork.com/2027-channelpro-defend-dallas/</t>
@@ -2789,6 +2778,7 @@
           <t>San Francisco</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>Salesforce</t>
@@ -2799,6 +2789,8 @@
           <t>Host</t>
         </is>
       </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" s="3" t="inlineStr">
         <is>
           <t>https://www.salesforce.com/dreamforce/</t>
@@ -2830,11 +2822,16 @@
           <t>Virtual</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>Virtual</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" s="3" t="inlineStr">
         <is>
           <t>https://events.channelpronetwork.com/channelpro-deep-dive-the-ai-powered-msp/</t>

</xml_diff>

<commit_message>
Publish tracker_all.csv (Year column) and per-year CSVs through 2030
One query on tracker_all.csv never needs touching when a new year starts; empty 2028-2030 files exist so per-year sheets keep working too.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TLMW817qEmLPfhM4KiByCq
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -1541,8 +1541,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
       <c r="L22" s="3" t="inlineStr">
         <is>
           <t>https://luma.com/agentsinnyc</t>
@@ -1657,7 +1655,6 @@
       <c r="C25" s="2" t="n">
         <v>46338</v>
       </c>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>Seattle</t>
@@ -1678,9 +1675,6 @@
           <t>AWS</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
       <c r="L25" s="3" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/saasify-partner-central-agentic-workshop-tickets-2003698327636</t>
@@ -1727,13 +1721,11 @@
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
           <t>Seattle Data, AI &amp; Security</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
       <c r="L26" s="3" t="inlineStr">
         <is>
           <t>https://www.meetup.com/seattledataaiandsecurity/events/316481475/</t>
@@ -1805,7 +1797,6 @@
       <c r="C28" s="2" t="n">
         <v>46343</v>
       </c>
-      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
           <t>Bay Area</t>
@@ -1826,9 +1817,6 @@
           <t>AWS</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
       <c r="L28" s="3" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/saasify-partner-central-agentic-workshop-tickets-2003695905391</t>
@@ -1875,9 +1863,6 @@
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
       <c r="L29" s="3" t="inlineStr">
         <is>
           <t>https://www.joincatalyst.com/catalyst-breakfast-at-microsoft-ignite</t>
@@ -2001,16 +1986,11 @@
           <t>Virtual</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
           <t>Virtual</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
       <c r="L32" s="3" t="inlineStr">
         <is>
           <t>https://www.channelmarketingassociation.com/industry-events</t>
@@ -2032,22 +2012,16 @@
         <v>46365</v>
       </c>
       <c r="C33" s="2" t="n"/>
-      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
           <t>New York</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
       <c r="L33" s="3" t="inlineStr">
         <is>
           <t>https://themspsummit.com/msp-summit-ai-symposium/</t>
@@ -2084,7 +2058,6 @@
           <t>Seattle</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -2095,8 +2068,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
       <c r="L34" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/seattle27/citylanding/page/cityhome</t>
@@ -2252,7 +2223,6 @@
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -2263,8 +2233,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymemumbai/page/notifyme</t>
@@ -2301,7 +2269,6 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -2312,8 +2279,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymebengaluru/page/notifyme</t>
@@ -2345,16 +2310,11 @@
           <t>Virtual</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>Virtual</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" s="3" t="inlineStr">
         <is>
           <t>https://events.channelpronetwork.com/channelpro-deep-dive-cybersecurity-in-the-age-of-ai/</t>
@@ -2388,12 +2348,6 @@
           <t>Texas</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" s="3" t="inlineStr">
         <is>
           <t>https://event.thechannelco.com/xchange-march/</t>
@@ -2430,7 +2384,6 @@
           <t>New York City</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -2441,8 +2394,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymenyc/page/notifyme</t>
@@ -2474,16 +2425,11 @@
           <t>Virtual</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>Virtual</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
       <c r="L7" s="3" t="inlineStr">
         <is>
           <t>https://events.channelpronetwork.com/channelpro-deep-dive-perfecting-your-tool-stack/</t>
@@ -2517,12 +2463,6 @@
           <t>Texas</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" s="3" t="inlineStr">
         <is>
           <t>https://www.channelmarketingassociation.com/Global-Summit-2027</t>
@@ -2554,16 +2494,11 @@
           <t>Virtual</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>Virtual</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" s="3" t="inlineStr">
         <is>
           <t>https://events.channelpronetwork.com/channelpro-deep-dive-the-most-profitable-cybersecurity-services-in-2027/</t>
@@ -2600,7 +2535,6 @@
           <t>Houston</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>Microsoft</t>
@@ -2611,8 +2545,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
       <c r="L10" s="3" t="inlineStr">
         <is>
           <t>https://aitour.microsoft.com/flow/microsoft/tour/notifymehouston/page/notifyme</t>
@@ -2646,8 +2578,6 @@
           <t>Bay Area</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>Databricks</t>
@@ -2658,8 +2588,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" s="3" t="inlineStr">
         <is>
           <t>https://www.databricks.com/dataaisummit/agenda</t>
@@ -2691,16 +2619,11 @@
           <t>Virtual</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>Virtual</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
       <c r="L12" s="3" t="inlineStr">
         <is>
           <t>https://events.channelpronetwork.com/channelpro-deep-dive-where-the-next-wave-of-msp-revenue-is-coming-from/</t>
@@ -2734,12 +2657,6 @@
           <t>Texas</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
       <c r="L13" s="3" t="inlineStr">
         <is>
           <t>https://events.channelpronetwork.com/2027-channelpro-defend-dallas/</t>
@@ -2778,7 +2695,6 @@
           <t>San Francisco</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>Salesforce</t>
@@ -2789,8 +2705,6 @@
           <t>Host</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
       <c r="L14" s="3" t="inlineStr">
         <is>
           <t>https://www.salesforce.com/dreamforce/</t>
@@ -2822,16 +2736,11 @@
           <t>Virtual</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>Virtual</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" s="3" t="inlineStr">
         <is>
           <t>https://events.channelpronetwork.com/channelpro-deep-dive-the-ai-powered-msp/</t>

</xml_diff>